<commit_message>
#4 Updated Client BOM
</commit_message>
<xml_diff>
--- a/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
+++ b/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1341" uniqueCount="718">
   <si>
     <t>#</t>
   </si>
@@ -2181,6 +2181,12 @@
   </si>
   <si>
     <t>IC RS232 LINE DVR/RCVR 16-SOIC</t>
+  </si>
+  <si>
+    <t>1.8 3dBi Vertical 50W - Antennas ROHS</t>
+  </si>
+  <si>
+    <t>BWGSMJWX105-7KJ</t>
   </si>
 </sst>
 </file>
@@ -8983,7 +8989,7 @@
         <v>6</v>
       </c>
       <c r="K132" s="12">
-        <f t="shared" ref="K132:K160" si="11">3*J132</f>
+        <f t="shared" ref="K132:K161" si="11">3*J132</f>
         <v>18</v>
       </c>
       <c r="L132" s="19" t="s">
@@ -10286,7 +10292,7 @@
       </c>
       <c r="O160" s="12"/>
     </row>
-    <row r="161" spans="2:19" ht="15.75" thickBot="1">
+    <row r="161" spans="2:19" ht="24.75" thickBot="1">
       <c r="B161" s="10">
         <f t="shared" ref="B161:B167" si="12">ROW(B161)-ROW($B$2)</f>
         <v>159</v>
@@ -10297,18 +10303,35 @@
       <c r="D161" s="12" t="s">
         <v>683</v>
       </c>
-      <c r="E161" s="13"/>
-      <c r="F161" s="15"/>
-      <c r="G161" s="13"/>
-      <c r="H161" s="12"/>
+      <c r="E161" s="13" t="s">
+        <v>716</v>
+      </c>
+      <c r="F161" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G161" s="13" t="s">
+        <v>717</v>
+      </c>
+      <c r="H161" s="12" t="s">
+        <v>249</v>
+      </c>
       <c r="I161" s="13"/>
-      <c r="J161" s="12"/>
-      <c r="K161" s="12"/>
-      <c r="L161" s="19"/>
-      <c r="M161" s="18"/>
+      <c r="J161" s="12">
+        <v>1</v>
+      </c>
+      <c r="K161" s="12">
+        <f t="shared" si="11"/>
+        <v>3</v>
+      </c>
+      <c r="L161" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="M161" s="18">
+        <v>1.0093000000000001</v>
+      </c>
       <c r="N161" s="18">
         <f>M161*K161</f>
-        <v>0</v>
+        <v>3.0279000000000003</v>
       </c>
       <c r="O161" s="12"/>
     </row>
@@ -10546,7 +10569,7 @@
       </c>
       <c r="N168" s="43">
         <f>SUM(N3:N167)</f>
-        <v>767.79249000000004</v>
+        <v>770.82039000000009</v>
       </c>
     </row>
     <row r="169" spans="2:19" ht="15.75" thickBot="1">
@@ -10555,7 +10578,7 @@
       </c>
       <c r="N169" s="45">
         <f>N168/3</f>
-        <v>255.93083000000001</v>
+        <v>256.94013000000001</v>
       </c>
     </row>
   </sheetData>
@@ -10722,6 +10745,7 @@
     <hyperlink ref="L56" r:id="rId157"/>
     <hyperlink ref="L71" r:id="rId158"/>
     <hyperlink ref="L134" r:id="rId159"/>
+    <hyperlink ref="L161" r:id="rId160"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
#4 eSpark BOM Updated.
</commit_message>
<xml_diff>
--- a/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
+++ b/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1341" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1333" uniqueCount="715">
   <si>
     <t>#</t>
   </si>
@@ -1420,9 +1420,6 @@
     <t>R56</t>
   </si>
   <si>
-    <t>R58, R66</t>
-  </si>
-  <si>
     <t>RES 12K OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -1571,15 +1568,6 @@
   </si>
   <si>
     <t>3K</t>
-  </si>
-  <si>
-    <t>R198</t>
-  </si>
-  <si>
-    <t>RES SMD 12K OHM 1% 1/5W 0402</t>
-  </si>
-  <si>
-    <t>RCS040212K0FKED</t>
   </si>
   <si>
     <t>R201, R202</t>
@@ -2187,6 +2175,9 @@
   </si>
   <si>
     <t>BWGSMJWX105-7KJ</t>
+  </si>
+  <si>
+    <t>R58, R66, R98</t>
   </si>
 </sst>
 </file>
@@ -2923,7 +2914,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S169"/>
+  <dimension ref="A1:S168"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="4.5703125" style="4" customWidth="1"/>
@@ -3047,7 +3038,7 @@
       </c>
       <c r="N3" s="18">
         <f>M3*K3</f>
-        <v>3.1137000000000001</v>
+        <v>3.1136999999999997</v>
       </c>
       <c r="O3" s="12"/>
     </row>
@@ -3093,7 +3084,7 @@
       </c>
       <c r="N4" s="18">
         <f t="shared" ref="N4:N15" si="2">M4*K4</f>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O4" s="15"/>
     </row>
@@ -3185,7 +3176,7 @@
       </c>
       <c r="N6" s="18">
         <f t="shared" si="2"/>
-        <v>1.74</v>
+        <v>1.7399999999999998</v>
       </c>
       <c r="O6" s="15"/>
     </row>
@@ -3277,7 +3268,7 @@
       </c>
       <c r="N8" s="18">
         <f t="shared" si="2"/>
-        <v>2.52</v>
+        <v>2.5200000000000005</v>
       </c>
       <c r="O8" s="15"/>
     </row>
@@ -3323,7 +3314,7 @@
       </c>
       <c r="N9" s="18">
         <f t="shared" si="2"/>
-        <v>2.0760000000000001</v>
+        <v>2.0759999999999996</v>
       </c>
       <c r="O9" s="12"/>
     </row>
@@ -3553,7 +3544,7 @@
       </c>
       <c r="N14" s="18">
         <f t="shared" si="2"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O14" s="15"/>
     </row>
@@ -3599,7 +3590,7 @@
       </c>
       <c r="N15" s="18">
         <f t="shared" si="2"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O15" s="12"/>
     </row>
@@ -3645,7 +3636,7 @@
       </c>
       <c r="N16" s="18">
         <f t="shared" ref="N16:N29" si="3">M16*K16</f>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O16" s="15"/>
     </row>
@@ -3737,7 +3728,7 @@
       </c>
       <c r="N18" s="18">
         <f t="shared" si="3"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O18" s="15"/>
     </row>
@@ -3783,7 +3774,7 @@
       </c>
       <c r="N19" s="18">
         <f t="shared" si="3"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O19" s="12"/>
     </row>
@@ -3875,7 +3866,7 @@
       </c>
       <c r="N21" s="18">
         <f t="shared" si="3"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O21" s="12"/>
     </row>
@@ -4013,7 +4004,7 @@
       </c>
       <c r="N24" s="18">
         <f t="shared" si="3"/>
-        <v>8.1</v>
+        <v>8.1000000000000014</v>
       </c>
       <c r="O24" s="15"/>
     </row>
@@ -4243,7 +4234,7 @@
       </c>
       <c r="N29" s="18">
         <f t="shared" si="3"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O29" s="12"/>
     </row>
@@ -4289,7 +4280,7 @@
       </c>
       <c r="N30" s="18">
         <f t="shared" ref="N30:N39" si="4">M30*K30</f>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O30" s="15"/>
     </row>
@@ -4381,7 +4372,7 @@
       </c>
       <c r="N32" s="18">
         <f t="shared" si="4"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O32" s="15"/>
     </row>
@@ -4427,7 +4418,7 @@
       </c>
       <c r="N33" s="18">
         <f t="shared" si="4"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O33" s="12"/>
     </row>
@@ -4519,7 +4510,7 @@
       </c>
       <c r="N35" s="18">
         <f t="shared" si="4"/>
-        <v>0.37559999999999999</v>
+        <v>0.37560000000000004</v>
       </c>
       <c r="O35" s="12"/>
     </row>
@@ -4565,7 +4556,7 @@
       </c>
       <c r="N36" s="18">
         <f t="shared" si="4"/>
-        <v>1.1100000000000001</v>
+        <v>1.1099999999999999</v>
       </c>
       <c r="O36" s="15"/>
     </row>
@@ -4887,7 +4878,7 @@
       </c>
       <c r="N43" s="18">
         <f t="shared" si="6"/>
-        <v>4.9800000000000004</v>
+        <v>4.9799999999999995</v>
       </c>
       <c r="O43" s="12"/>
     </row>
@@ -5025,7 +5016,7 @@
       </c>
       <c r="N46" s="18">
         <f t="shared" si="6"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O46" s="15"/>
     </row>
@@ -5209,7 +5200,7 @@
       </c>
       <c r="N50" s="18">
         <f t="shared" si="6"/>
-        <v>3.78</v>
+        <v>3.7800000000000002</v>
       </c>
       <c r="O50" s="12"/>
     </row>
@@ -5439,7 +5430,7 @@
       </c>
       <c r="N55" s="18">
         <f t="shared" si="6"/>
-        <v>1.2890999999999999</v>
+        <v>1.2891000000000001</v>
       </c>
       <c r="O55" s="15"/>
     </row>
@@ -5450,22 +5441,22 @@
         <v>54</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>711</v>
+        <v>707</v>
       </c>
       <c r="D56" s="15" t="s">
         <v>248</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>712</v>
+        <v>708</v>
       </c>
       <c r="F56" s="15" t="s">
         <v>111</v>
       </c>
       <c r="G56" s="15" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="H56" s="15" t="s">
-        <v>713</v>
+        <v>709</v>
       </c>
       <c r="I56" s="16" t="s">
         <v>150</v>
@@ -5531,14 +5522,14 @@
       </c>
       <c r="N57" s="18">
         <f t="shared" si="7"/>
-        <v>3.3</v>
+        <v>3.3000000000000003</v>
       </c>
       <c r="O57" s="12"/>
     </row>
     <row r="58" spans="1:15" ht="60.75" thickBot="1">
       <c r="A58" s="5"/>
       <c r="B58" s="10">
-        <f t="shared" ref="B58:B159" si="8">ROW(B58)-ROW($B$2)</f>
+        <f t="shared" ref="B58:B158" si="8">ROW(B58)-ROW($B$2)</f>
         <v>56</v>
       </c>
       <c r="C58" s="14" t="s">
@@ -5715,7 +5706,7 @@
       </c>
       <c r="N61" s="18">
         <f t="shared" si="7"/>
-        <v>1.38</v>
+        <v>1.3800000000000001</v>
       </c>
       <c r="O61" s="12"/>
     </row>
@@ -5807,7 +5798,7 @@
       </c>
       <c r="N63" s="18">
         <f t="shared" si="7"/>
-        <v>15.322800000000001</v>
+        <v>15.322799999999999</v>
       </c>
       <c r="O63" s="12"/>
     </row>
@@ -5945,7 +5936,7 @@
       </c>
       <c r="N66" s="18">
         <f t="shared" si="7"/>
-        <v>1.0169999999999999</v>
+        <v>1.0170000000000001</v>
       </c>
       <c r="O66" s="15"/>
     </row>
@@ -6026,7 +6017,7 @@
         <v>2</v>
       </c>
       <c r="K68" s="12">
-        <f t="shared" ref="K68:K131" si="9">3*J68</f>
+        <f t="shared" ref="K68:K130" si="9">3*J68</f>
         <v>6</v>
       </c>
       <c r="L68" s="19" t="s">
@@ -6129,7 +6120,7 @@
       </c>
       <c r="N70" s="18">
         <f t="shared" si="7"/>
-        <v>67.349999999999994</v>
+        <v>67.350000000000009</v>
       </c>
       <c r="O70" s="15"/>
     </row>
@@ -6140,7 +6131,7 @@
         <v>69</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="D71" s="15" t="s">
         <v>307</v>
@@ -6152,7 +6143,7 @@
         <v>111</v>
       </c>
       <c r="G71" s="15" t="s">
-        <v>709</v>
+        <v>705</v>
       </c>
       <c r="H71" s="15" t="s">
         <v>53</v>
@@ -6267,7 +6258,7 @@
       </c>
       <c r="N73" s="18">
         <f t="shared" si="7"/>
-        <v>1.2</v>
+        <v>1.2000000000000002</v>
       </c>
       <c r="O73" s="12"/>
     </row>
@@ -6497,7 +6488,7 @@
       </c>
       <c r="N78" s="18">
         <f t="shared" si="7"/>
-        <v>1.05</v>
+        <v>1.0499999999999998</v>
       </c>
       <c r="O78" s="15"/>
     </row>
@@ -6543,7 +6534,7 @@
       </c>
       <c r="N79" s="18">
         <f t="shared" si="7"/>
-        <v>0.9</v>
+        <v>0.89999999999999991</v>
       </c>
       <c r="O79" s="12"/>
     </row>
@@ -6727,7 +6718,7 @@
       </c>
       <c r="N83" s="18">
         <f t="shared" si="7"/>
-        <v>0.54479999999999995</v>
+        <v>0.54480000000000006</v>
       </c>
       <c r="O83" s="12"/>
     </row>
@@ -6773,7 +6764,7 @@
       </c>
       <c r="N84" s="18">
         <f t="shared" si="7"/>
-        <v>1.74</v>
+        <v>1.7399999999999998</v>
       </c>
       <c r="O84" s="15"/>
     </row>
@@ -6819,7 +6810,7 @@
       </c>
       <c r="N85" s="18">
         <f t="shared" si="7"/>
-        <v>6.15</v>
+        <v>6.1499999999999995</v>
       </c>
       <c r="O85" s="12"/>
     </row>
@@ -7283,7 +7274,7 @@
       </c>
       <c r="N95" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O95" s="12"/>
     </row>
@@ -7375,7 +7366,7 @@
       </c>
       <c r="N97" s="18">
         <f t="shared" si="7"/>
-        <v>0.40389000000000003</v>
+        <v>0.40388999999999997</v>
       </c>
       <c r="O97" s="12"/>
     </row>
@@ -7467,7 +7458,7 @@
       </c>
       <c r="N99" s="18">
         <f t="shared" si="7"/>
-        <v>1.4039999999999999</v>
+        <v>1.4040000000000001</v>
       </c>
       <c r="O99" s="12"/>
     </row>
@@ -7605,7 +7596,7 @@
       </c>
       <c r="N102" s="18">
         <f t="shared" si="7"/>
-        <v>5.7000000000000002E-2</v>
+        <v>5.6999999999999995E-2</v>
       </c>
       <c r="O102" s="15"/>
     </row>
@@ -7651,7 +7642,7 @@
       </c>
       <c r="N103" s="18">
         <f t="shared" si="7"/>
-        <v>0.22500000000000001</v>
+        <v>0.22499999999999998</v>
       </c>
       <c r="O103" s="12"/>
     </row>
@@ -7697,7 +7688,7 @@
       </c>
       <c r="N104" s="18">
         <f t="shared" si="7"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O104" s="15"/>
     </row>
@@ -7743,7 +7734,7 @@
       </c>
       <c r="N105" s="18">
         <f t="shared" si="7"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O105" s="12"/>
     </row>
@@ -7789,7 +7780,7 @@
       </c>
       <c r="N106" s="18">
         <f t="shared" si="7"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O106" s="15"/>
     </row>
@@ -7853,29 +7844,29 @@
         <v>386</v>
       </c>
       <c r="D108" s="15" t="s">
+        <v>714</v>
+      </c>
+      <c r="E108" s="16" t="s">
         <v>462</v>
-      </c>
-      <c r="E108" s="16" t="s">
-        <v>463</v>
       </c>
       <c r="F108" s="15" t="s">
         <v>389</v>
       </c>
       <c r="G108" s="16" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H108" s="15" t="s">
         <v>19</v>
       </c>
       <c r="I108" s="16" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="J108" s="15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K108" s="12">
         <f t="shared" si="9"/>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="L108" s="19" t="s">
         <v>21</v>
@@ -7885,7 +7876,7 @@
       </c>
       <c r="N108" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="O108" s="15"/>
     </row>
@@ -7899,22 +7890,22 @@
         <v>386</v>
       </c>
       <c r="D109" s="12" t="s">
+        <v>465</v>
+      </c>
+      <c r="E109" s="13" t="s">
         <v>466</v>
-      </c>
-      <c r="E109" s="13" t="s">
-        <v>467</v>
       </c>
       <c r="F109" s="12" t="s">
         <v>389</v>
       </c>
       <c r="G109" s="13" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H109" s="12" t="s">
         <v>19</v>
       </c>
       <c r="I109" s="13" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="J109" s="12">
         <v>2</v>
@@ -7931,7 +7922,7 @@
       </c>
       <c r="N109" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O109" s="12"/>
     </row>
@@ -7945,7 +7936,7 @@
         <v>386</v>
       </c>
       <c r="D110" s="23" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E110" s="24" t="s">
         <v>426</v>
@@ -7992,19 +7983,19 @@
         <v>386</v>
       </c>
       <c r="D111" s="12" t="s">
+        <v>470</v>
+      </c>
+      <c r="E111" s="13" t="s">
         <v>471</v>
-      </c>
-      <c r="E111" s="13" t="s">
-        <v>472</v>
       </c>
       <c r="F111" s="12" t="s">
         <v>415</v>
       </c>
       <c r="G111" s="13" t="s">
+        <v>472</v>
+      </c>
+      <c r="H111" s="12" t="s">
         <v>473</v>
-      </c>
-      <c r="H111" s="12" t="s">
-        <v>474</v>
       </c>
       <c r="I111" s="13" t="s">
         <v>407</v>
@@ -8024,7 +8015,7 @@
       </c>
       <c r="N111" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O111" s="12"/>
     </row>
@@ -8038,22 +8029,22 @@
         <v>386</v>
       </c>
       <c r="D112" s="15" t="s">
+        <v>474</v>
+      </c>
+      <c r="E112" s="16" t="s">
         <v>475</v>
-      </c>
-      <c r="E112" s="16" t="s">
-        <v>476</v>
       </c>
       <c r="F112" s="15" t="s">
         <v>415</v>
       </c>
       <c r="G112" s="16" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="H112" s="15" t="s">
         <v>19</v>
       </c>
       <c r="I112" s="16" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="J112" s="15">
         <v>2</v>
@@ -8070,7 +8061,7 @@
       </c>
       <c r="N112" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O112" s="15"/>
     </row>
@@ -8084,16 +8075,16 @@
         <v>386</v>
       </c>
       <c r="D113" s="12" t="s">
+        <v>478</v>
+      </c>
+      <c r="E113" s="13" t="s">
         <v>479</v>
-      </c>
-      <c r="E113" s="13" t="s">
-        <v>480</v>
       </c>
       <c r="F113" s="12" t="s">
         <v>415</v>
       </c>
       <c r="G113" s="13" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="H113" s="12" t="s">
         <v>19</v>
@@ -8130,22 +8121,22 @@
         <v>386</v>
       </c>
       <c r="D114" s="15" t="s">
+        <v>481</v>
+      </c>
+      <c r="E114" s="16" t="s">
         <v>482</v>
-      </c>
-      <c r="E114" s="16" t="s">
-        <v>483</v>
       </c>
       <c r="F114" s="15" t="s">
         <v>389</v>
       </c>
       <c r="G114" s="16" t="s">
+        <v>483</v>
+      </c>
+      <c r="H114" s="15" t="s">
+        <v>473</v>
+      </c>
+      <c r="I114" s="16" t="s">
         <v>484</v>
-      </c>
-      <c r="H114" s="15" t="s">
-        <v>474</v>
-      </c>
-      <c r="I114" s="16" t="s">
-        <v>485</v>
       </c>
       <c r="J114" s="15">
         <v>2</v>
@@ -8176,22 +8167,22 @@
         <v>386</v>
       </c>
       <c r="D115" s="31" t="s">
+        <v>485</v>
+      </c>
+      <c r="E115" s="32" t="s">
         <v>486</v>
-      </c>
-      <c r="E115" s="32" t="s">
-        <v>487</v>
       </c>
       <c r="F115" s="31" t="s">
         <v>389</v>
       </c>
       <c r="G115" s="32" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="H115" s="31" t="s">
         <v>19</v>
       </c>
       <c r="I115" s="32" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="J115" s="31">
         <v>8</v>
@@ -8225,7 +8216,7 @@
         <v>386</v>
       </c>
       <c r="D116" s="33" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="E116" s="34" t="s">
         <v>409</v>
@@ -8240,7 +8231,7 @@
         <v>19</v>
       </c>
       <c r="I116" s="34" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="J116" s="33">
         <v>8</v>
@@ -8274,22 +8265,22 @@
         <v>386</v>
       </c>
       <c r="D117" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="E117" s="13" t="s">
         <v>492</v>
-      </c>
-      <c r="E117" s="13" t="s">
-        <v>493</v>
       </c>
       <c r="F117" s="12" t="s">
         <v>389</v>
       </c>
       <c r="G117" s="13" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="H117" s="12" t="s">
         <v>19</v>
       </c>
       <c r="I117" s="13" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="J117" s="12">
         <v>2</v>
@@ -8306,7 +8297,7 @@
       </c>
       <c r="N117" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O117" s="12"/>
     </row>
@@ -8320,22 +8311,22 @@
         <v>386</v>
       </c>
       <c r="D118" s="15" t="s">
+        <v>495</v>
+      </c>
+      <c r="E118" s="16" t="s">
         <v>496</v>
-      </c>
-      <c r="E118" s="16" t="s">
-        <v>497</v>
       </c>
       <c r="F118" s="15" t="s">
         <v>389</v>
       </c>
       <c r="G118" s="16" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="H118" s="15" t="s">
         <v>19</v>
       </c>
       <c r="I118" s="16" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="J118" s="15">
         <v>2</v>
@@ -8352,7 +8343,7 @@
       </c>
       <c r="N118" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O118" s="15"/>
     </row>
@@ -8363,19 +8354,19 @@
         <v>117</v>
       </c>
       <c r="C119" s="11" t="s">
+        <v>499</v>
+      </c>
+      <c r="D119" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="D119" s="12" t="s">
+      <c r="E119" s="13" t="s">
         <v>501</v>
-      </c>
-      <c r="E119" s="13" t="s">
-        <v>502</v>
       </c>
       <c r="F119" s="12" t="s">
         <v>389</v>
       </c>
       <c r="G119" s="13" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="H119" s="12" t="s">
         <v>19</v>
@@ -8398,7 +8389,7 @@
       </c>
       <c r="N119" s="18">
         <f t="shared" si="7"/>
-        <v>0.6</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O119" s="12"/>
     </row>
@@ -8409,25 +8400,25 @@
         <v>118</v>
       </c>
       <c r="C120" s="14" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="D120" s="15" t="s">
+        <v>503</v>
+      </c>
+      <c r="E120" s="16" t="s">
         <v>504</v>
-      </c>
-      <c r="E120" s="16" t="s">
-        <v>505</v>
       </c>
       <c r="F120" s="15" t="s">
         <v>389</v>
       </c>
       <c r="G120" s="16" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="H120" s="15" t="s">
         <v>19</v>
       </c>
       <c r="I120" s="16" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="J120" s="15">
         <v>2</v>
@@ -8443,8 +8434,8 @@
         <v>0.1</v>
       </c>
       <c r="N120" s="18">
-        <f t="shared" ref="N120:N160" si="10">M120*K120</f>
-        <v>0.6</v>
+        <f t="shared" ref="N120:N159" si="10">M120*K120</f>
+        <v>0.60000000000000009</v>
       </c>
       <c r="O120" s="15"/>
     </row>
@@ -8458,7 +8449,7 @@
         <v>386</v>
       </c>
       <c r="D121" s="26" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="E121" s="27" t="s">
         <v>388</v>
@@ -8508,22 +8499,22 @@
         <v>386</v>
       </c>
       <c r="D122" s="15" t="s">
+        <v>508</v>
+      </c>
+      <c r="E122" s="16" t="s">
         <v>509</v>
-      </c>
-      <c r="E122" s="16" t="s">
-        <v>510</v>
       </c>
       <c r="F122" s="15" t="s">
         <v>389</v>
       </c>
       <c r="G122" s="16" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H122" s="15" t="s">
         <v>19</v>
       </c>
       <c r="I122" s="16" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="J122" s="15">
         <v>1</v>
@@ -8540,89 +8531,89 @@
       </c>
       <c r="N122" s="18">
         <f t="shared" si="10"/>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="O122" s="15"/>
     </row>
     <row r="123" spans="1:19" ht="15.75" thickBot="1">
       <c r="A123" s="5"/>
       <c r="B123" s="10">
-        <f>ROW(B123)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>121</v>
       </c>
-      <c r="C123" s="11" t="s">
+      <c r="C123" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="D123" s="12" t="s">
+      <c r="D123" s="15" t="s">
+        <v>512</v>
+      </c>
+      <c r="E123" s="16" t="s">
         <v>513</v>
       </c>
-      <c r="E123" s="13" t="s">
+      <c r="F123" s="15" t="s">
+        <v>415</v>
+      </c>
+      <c r="G123" s="16" t="s">
         <v>514</v>
       </c>
-      <c r="F123" s="12" t="s">
-        <v>389</v>
-      </c>
-      <c r="G123" s="13" t="s">
+      <c r="H123" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="I123" s="16" t="s">
         <v>515</v>
       </c>
-      <c r="H123" s="12" t="s">
-        <v>474</v>
-      </c>
-      <c r="I123" s="13" t="s">
-        <v>465</v>
-      </c>
-      <c r="J123" s="12">
-        <v>1</v>
+      <c r="J123" s="15">
+        <v>2</v>
       </c>
       <c r="K123" s="12">
         <f t="shared" si="9"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L123" s="19" t="s">
         <v>21</v>
       </c>
       <c r="M123" s="18">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="N123" s="18">
         <f t="shared" si="10"/>
-        <v>0.33</v>
-      </c>
-      <c r="O123" s="12"/>
+        <v>0.60000000000000009</v>
+      </c>
+      <c r="O123" s="15"/>
     </row>
     <row r="124" spans="1:19" ht="15.75" thickBot="1">
       <c r="A124" s="5"/>
       <c r="B124" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B124)-ROW($B$2)</f>
         <v>122</v>
       </c>
-      <c r="C124" s="14" t="s">
+      <c r="C124" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="D124" s="15" t="s">
+      <c r="D124" s="12" t="s">
         <v>516</v>
       </c>
-      <c r="E124" s="16" t="s">
+      <c r="E124" s="13" t="s">
         <v>517</v>
       </c>
-      <c r="F124" s="15" t="s">
-        <v>415</v>
-      </c>
-      <c r="G124" s="16" t="s">
+      <c r="F124" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="G124" s="13" t="s">
         <v>518</v>
       </c>
-      <c r="H124" s="15" t="s">
+      <c r="H124" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I124" s="16" t="s">
+      <c r="I124" s="13" t="s">
         <v>519</v>
       </c>
-      <c r="J124" s="15">
-        <v>2</v>
+      <c r="J124" s="12">
+        <v>1</v>
       </c>
       <c r="K124" s="12">
         <f t="shared" si="9"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L124" s="19" t="s">
         <v>21</v>
@@ -8632,38 +8623,38 @@
       </c>
       <c r="N124" s="18">
         <f t="shared" si="10"/>
-        <v>0.6</v>
-      </c>
-      <c r="O124" s="15"/>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="O124" s="12"/>
     </row>
     <row r="125" spans="1:19" ht="15.75" thickBot="1">
       <c r="A125" s="5"/>
       <c r="B125" s="10">
-        <f>ROW(B125)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>123</v>
       </c>
-      <c r="C125" s="11" t="s">
+      <c r="C125" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="D125" s="12" t="s">
+      <c r="D125" s="15" t="s">
         <v>520</v>
       </c>
-      <c r="E125" s="13" t="s">
+      <c r="E125" s="16" t="s">
         <v>521</v>
       </c>
-      <c r="F125" s="12" t="s">
+      <c r="F125" s="15" t="s">
         <v>389</v>
       </c>
-      <c r="G125" s="13" t="s">
+      <c r="G125" s="16" t="s">
         <v>522</v>
       </c>
-      <c r="H125" s="12" t="s">
+      <c r="H125" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="I125" s="13" t="s">
+      <c r="I125" s="16" t="s">
         <v>523</v>
       </c>
-      <c r="J125" s="12">
+      <c r="J125" s="15">
         <v>1</v>
       </c>
       <c r="K125" s="12">
@@ -8678,38 +8669,38 @@
       </c>
       <c r="N125" s="18">
         <f t="shared" si="10"/>
-        <v>0.3</v>
-      </c>
-      <c r="O125" s="12"/>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="O125" s="15"/>
     </row>
     <row r="126" spans="1:19" ht="15.75" thickBot="1">
       <c r="A126" s="5"/>
       <c r="B126" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B126)-ROW($B$2)</f>
         <v>124</v>
       </c>
-      <c r="C126" s="14" t="s">
+      <c r="C126" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="D126" s="15" t="s">
+      <c r="D126" s="12" t="s">
         <v>524</v>
       </c>
-      <c r="E126" s="16" t="s">
+      <c r="E126" s="13" t="s">
         <v>525</v>
       </c>
-      <c r="F126" s="15" t="s">
+      <c r="F126" s="12" t="s">
         <v>389</v>
       </c>
-      <c r="G126" s="16" t="s">
+      <c r="G126" s="13" t="s">
         <v>526</v>
       </c>
-      <c r="H126" s="15" t="s">
+      <c r="H126" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I126" s="16" t="s">
+      <c r="I126" s="13" t="s">
         <v>527</v>
       </c>
-      <c r="J126" s="15">
+      <c r="J126" s="12">
         <v>1</v>
       </c>
       <c r="K126" s="12">
@@ -8724,38 +8715,38 @@
       </c>
       <c r="N126" s="18">
         <f t="shared" si="10"/>
-        <v>0.3</v>
-      </c>
-      <c r="O126" s="15"/>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="O126" s="12"/>
     </row>
     <row r="127" spans="1:19" ht="15.75" thickBot="1">
       <c r="A127" s="5"/>
       <c r="B127" s="10">
-        <f>ROW(B127)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>125</v>
       </c>
-      <c r="C127" s="11" t="s">
+      <c r="C127" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="D127" s="12" t="s">
+      <c r="D127" s="15" t="s">
         <v>528</v>
       </c>
-      <c r="E127" s="13" t="s">
+      <c r="E127" s="16" t="s">
         <v>529</v>
       </c>
-      <c r="F127" s="12" t="s">
+      <c r="F127" s="15" t="s">
         <v>389</v>
       </c>
-      <c r="G127" s="13" t="s">
+      <c r="G127" s="16" t="s">
         <v>530</v>
       </c>
-      <c r="H127" s="12" t="s">
+      <c r="H127" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="I127" s="13" t="s">
+      <c r="I127" s="16" t="s">
         <v>531</v>
       </c>
-      <c r="J127" s="12">
+      <c r="J127" s="15">
         <v>1</v>
       </c>
       <c r="K127" s="12">
@@ -8770,89 +8761,89 @@
       </c>
       <c r="N127" s="18">
         <f t="shared" si="10"/>
-        <v>0.3</v>
-      </c>
-      <c r="O127" s="12"/>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="O127" s="15"/>
     </row>
     <row r="128" spans="1:19" ht="15.75" thickBot="1">
       <c r="A128" s="5"/>
       <c r="B128" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B128)-ROW($B$2)</f>
         <v>126</v>
       </c>
-      <c r="C128" s="14" t="s">
+      <c r="C128" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="D128" s="15" t="s">
+      <c r="D128" s="12" t="s">
         <v>532</v>
       </c>
-      <c r="E128" s="16" t="s">
+      <c r="E128" s="13" t="s">
         <v>533</v>
       </c>
-      <c r="F128" s="15" t="s">
+      <c r="F128" s="12" t="s">
         <v>389</v>
       </c>
-      <c r="G128" s="16" t="s">
+      <c r="G128" s="13" t="s">
         <v>534</v>
       </c>
-      <c r="H128" s="15" t="s">
+      <c r="H128" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I128" s="16" t="s">
-        <v>535</v>
-      </c>
-      <c r="J128" s="15">
-        <v>1</v>
+      <c r="I128" s="13" t="s">
+        <v>444</v>
+      </c>
+      <c r="J128" s="12">
+        <v>2</v>
       </c>
       <c r="K128" s="12">
         <f t="shared" si="9"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L128" s="19" t="s">
         <v>21</v>
       </c>
       <c r="M128" s="18">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="N128" s="18">
         <f t="shared" si="10"/>
-        <v>0.3</v>
-      </c>
-      <c r="O128" s="15"/>
+        <v>0.96</v>
+      </c>
+      <c r="O128" s="12"/>
     </row>
     <row r="129" spans="1:15" ht="15.75" thickBot="1">
       <c r="A129" s="5"/>
       <c r="B129" s="10">
-        <f>ROW(B129)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>127</v>
       </c>
-      <c r="C129" s="11" t="s">
+      <c r="C129" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="D129" s="12" t="s">
+      <c r="D129" s="15" t="s">
+        <v>535</v>
+      </c>
+      <c r="E129" s="16" t="s">
         <v>536</v>
       </c>
-      <c r="E129" s="13" t="s">
+      <c r="F129" s="15" t="s">
+        <v>389</v>
+      </c>
+      <c r="G129" s="16" t="s">
         <v>537</v>
       </c>
-      <c r="F129" s="12" t="s">
-        <v>389</v>
-      </c>
-      <c r="G129" s="13" t="s">
-        <v>538</v>
-      </c>
-      <c r="H129" s="12" t="s">
+      <c r="H129" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="I129" s="13" t="s">
-        <v>444</v>
-      </c>
-      <c r="J129" s="12">
-        <v>2</v>
+      <c r="I129" s="16" t="s">
+        <v>494</v>
+      </c>
+      <c r="J129" s="15">
+        <v>1</v>
       </c>
       <c r="K129" s="12">
         <f t="shared" si="9"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L129" s="19" t="s">
         <v>21</v>
@@ -8862,176 +8853,176 @@
       </c>
       <c r="N129" s="18">
         <f t="shared" si="10"/>
-        <v>0.96</v>
-      </c>
-      <c r="O129" s="12"/>
+        <v>0.48</v>
+      </c>
+      <c r="O129" s="15"/>
     </row>
     <row r="130" spans="1:15" ht="15.75" thickBot="1">
       <c r="A130" s="5"/>
       <c r="B130" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B130)-ROW($B$2)</f>
         <v>128</v>
       </c>
-      <c r="C130" s="14" t="s">
+      <c r="C130" s="11" t="s">
         <v>386</v>
       </c>
-      <c r="D130" s="15" t="s">
+      <c r="D130" s="12" t="s">
+        <v>538</v>
+      </c>
+      <c r="E130" s="13" t="s">
         <v>539</v>
       </c>
-      <c r="E130" s="16" t="s">
+      <c r="F130" s="12" t="s">
         <v>540</v>
       </c>
-      <c r="F130" s="15" t="s">
-        <v>389</v>
-      </c>
-      <c r="G130" s="16" t="s">
+      <c r="G130" s="13" t="s">
         <v>541</v>
       </c>
-      <c r="H130" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="I130" s="16" t="s">
-        <v>495</v>
-      </c>
-      <c r="J130" s="15">
-        <v>1</v>
+      <c r="H130" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="I130" s="13" t="s">
+        <v>420</v>
+      </c>
+      <c r="J130" s="12">
+        <v>2</v>
       </c>
       <c r="K130" s="12">
         <f t="shared" si="9"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L130" s="19" t="s">
         <v>21</v>
       </c>
       <c r="M130" s="18">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="N130" s="18">
         <f t="shared" si="10"/>
-        <v>0.48</v>
-      </c>
-      <c r="O130" s="15"/>
-    </row>
-    <row r="131" spans="1:15" ht="15.75" thickBot="1">
+        <v>0.89999999999999991</v>
+      </c>
+      <c r="O130" s="12"/>
+    </row>
+    <row r="131" spans="1:15" ht="36.75" thickBot="1">
       <c r="A131" s="5"/>
       <c r="B131" s="10">
-        <f>ROW(B131)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>129</v>
       </c>
-      <c r="C131" s="11" t="s">
-        <v>386</v>
-      </c>
-      <c r="D131" s="12" t="s">
-        <v>542</v>
-      </c>
-      <c r="E131" s="13" t="s">
+      <c r="C131" s="14" t="s">
         <v>543</v>
       </c>
-      <c r="F131" s="12" t="s">
+      <c r="D131" s="15" t="s">
         <v>544</v>
       </c>
-      <c r="G131" s="13" t="s">
+      <c r="E131" s="16" t="s">
         <v>545</v>
       </c>
-      <c r="H131" s="12" t="s">
+      <c r="F131" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G131" s="16" t="s">
         <v>546</v>
       </c>
-      <c r="I131" s="13" t="s">
-        <v>420</v>
-      </c>
-      <c r="J131" s="12">
-        <v>2</v>
+      <c r="H131" s="15" t="s">
+        <v>547</v>
+      </c>
+      <c r="I131" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="J131" s="15">
+        <v>6</v>
       </c>
       <c r="K131" s="12">
-        <f t="shared" si="9"/>
-        <v>6</v>
+        <f t="shared" ref="K131:K160" si="11">3*J131</f>
+        <v>18</v>
       </c>
       <c r="L131" s="19" t="s">
-        <v>21</v>
+        <v>114</v>
       </c>
       <c r="M131" s="18">
-        <v>0.15</v>
+        <v>6.9400000000000003E-2</v>
       </c>
       <c r="N131" s="18">
         <f t="shared" si="10"/>
-        <v>0.9</v>
-      </c>
-      <c r="O131" s="12"/>
-    </row>
-    <row r="132" spans="1:15" ht="36.75" thickBot="1">
+        <v>1.2492000000000001</v>
+      </c>
+      <c r="O131" s="15"/>
+    </row>
+    <row r="132" spans="1:15" ht="24.75" thickBot="1">
       <c r="A132" s="5"/>
       <c r="B132" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B132)-ROW($B$2)</f>
         <v>130</v>
       </c>
-      <c r="C132" s="14" t="s">
-        <v>547</v>
-      </c>
-      <c r="D132" s="15" t="s">
+      <c r="C132" s="11" t="s">
         <v>548</v>
       </c>
-      <c r="E132" s="16" t="s">
+      <c r="D132" s="12" t="s">
         <v>549</v>
       </c>
-      <c r="F132" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="G132" s="16" t="s">
+      <c r="E132" s="13" t="s">
         <v>550</v>
       </c>
-      <c r="H132" s="15" t="s">
+      <c r="F132" s="12" t="s">
         <v>551</v>
+      </c>
+      <c r="G132" s="13" t="s">
+        <v>552</v>
+      </c>
+      <c r="H132" s="12" t="s">
+        <v>553</v>
       </c>
       <c r="I132" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J132" s="15">
-        <v>6</v>
+      <c r="J132" s="12">
+        <v>1</v>
       </c>
       <c r="K132" s="12">
-        <f t="shared" ref="K132:K161" si="11">3*J132</f>
-        <v>18</v>
+        <f t="shared" si="11"/>
+        <v>3</v>
       </c>
       <c r="L132" s="19" t="s">
         <v>114</v>
       </c>
       <c r="M132" s="18">
-        <v>6.9400000000000003E-2</v>
+        <v>0.25340000000000001</v>
       </c>
       <c r="N132" s="18">
         <f t="shared" si="10"/>
-        <v>1.2492000000000001</v>
-      </c>
-      <c r="O132" s="15"/>
+        <v>0.76019999999999999</v>
+      </c>
+      <c r="O132" s="12"/>
     </row>
     <row r="133" spans="1:15" ht="24.75" thickBot="1">
       <c r="A133" s="5"/>
       <c r="B133" s="10">
-        <f>ROW(B133)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>131</v>
       </c>
       <c r="C133" s="11" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="D133" s="12" t="s">
-        <v>553</v>
-      </c>
-      <c r="E133" s="13" t="s">
         <v>554</v>
+      </c>
+      <c r="E133" s="12" t="s">
+        <v>711</v>
       </c>
       <c r="F133" s="12" t="s">
         <v>555</v>
       </c>
-      <c r="G133" s="13" t="s">
+      <c r="G133" s="12" t="s">
+        <v>706</v>
+      </c>
+      <c r="H133" s="12" t="s">
         <v>556</v>
-      </c>
-      <c r="H133" s="12" t="s">
-        <v>557</v>
       </c>
       <c r="I133" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J133" s="12">
+      <c r="J133" s="15">
         <v>1</v>
       </c>
       <c r="K133" s="12">
@@ -9039,229 +9030,229 @@
         <v>3</v>
       </c>
       <c r="L133" s="19" t="s">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="M133" s="18">
-        <v>0.25340000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="N133" s="18">
         <f t="shared" si="10"/>
-        <v>0.76019999999999999</v>
-      </c>
-      <c r="O133" s="12"/>
-    </row>
-    <row r="134" spans="1:15" ht="24.75" thickBot="1">
+        <v>4.5</v>
+      </c>
+      <c r="O133" s="40"/>
+    </row>
+    <row r="134" spans="1:15" ht="15.75" thickBot="1">
       <c r="A134" s="5"/>
       <c r="B134" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B134)-ROW($B$2)</f>
         <v>132</v>
       </c>
       <c r="C134" s="11" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="D134" s="12" t="s">
+        <v>557</v>
+      </c>
+      <c r="E134" s="13" t="s">
         <v>558</v>
-      </c>
-      <c r="E134" s="12" t="s">
-        <v>715</v>
       </c>
       <c r="F134" s="12" t="s">
         <v>559</v>
       </c>
-      <c r="G134" s="12" t="s">
-        <v>710</v>
+      <c r="G134" s="13" t="s">
+        <v>560</v>
       </c>
       <c r="H134" s="12" t="s">
-        <v>560</v>
+        <v>160</v>
       </c>
       <c r="I134" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J134" s="15">
-        <v>1</v>
+      <c r="J134" s="12">
+        <v>2</v>
       </c>
       <c r="K134" s="12">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L134" s="19" t="s">
         <v>21</v>
       </c>
       <c r="M134" s="18">
-        <v>1.5</v>
+        <v>0.46</v>
       </c>
       <c r="N134" s="18">
         <f t="shared" si="10"/>
-        <v>4.5</v>
-      </c>
-      <c r="O134" s="40"/>
-    </row>
-    <row r="135" spans="1:15" ht="15.75" thickBot="1">
+        <v>2.7600000000000002</v>
+      </c>
+      <c r="O134" s="12"/>
+    </row>
+    <row r="135" spans="1:15" ht="24.75" thickBot="1">
       <c r="A135" s="5"/>
       <c r="B135" s="10">
-        <f>ROW(B135)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>133</v>
       </c>
-      <c r="C135" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D135" s="12" t="s">
+      <c r="C135" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D135" s="15" t="s">
         <v>561</v>
       </c>
-      <c r="E135" s="13" t="s">
+      <c r="E135" s="16" t="s">
         <v>562</v>
       </c>
-      <c r="F135" s="12" t="s">
+      <c r="F135" s="15" t="s">
         <v>563</v>
       </c>
-      <c r="G135" s="13" t="s">
+      <c r="G135" s="16" t="s">
         <v>564</v>
       </c>
-      <c r="H135" s="12" t="s">
-        <v>160</v>
+      <c r="H135" s="15" t="s">
+        <v>556</v>
       </c>
       <c r="I135" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J135" s="12">
-        <v>2</v>
+      <c r="J135" s="15">
+        <v>1</v>
       </c>
       <c r="K135" s="12">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L135" s="19" t="s">
         <v>21</v>
       </c>
       <c r="M135" s="18">
-        <v>0.46</v>
+        <v>1.18</v>
       </c>
       <c r="N135" s="18">
         <f t="shared" si="10"/>
-        <v>2.76</v>
-      </c>
-      <c r="O135" s="12"/>
+        <v>3.54</v>
+      </c>
+      <c r="O135" s="15"/>
     </row>
     <row r="136" spans="1:15" ht="24.75" thickBot="1">
       <c r="A136" s="5"/>
       <c r="B136" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B136)-ROW($B$2)</f>
         <v>134</v>
       </c>
-      <c r="C136" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D136" s="15" t="s">
+      <c r="C136" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D136" s="12" t="s">
         <v>565</v>
       </c>
-      <c r="E136" s="16" t="s">
+      <c r="E136" s="13" t="s">
         <v>566</v>
       </c>
-      <c r="F136" s="15" t="s">
+      <c r="F136" s="12" t="s">
         <v>567</v>
       </c>
-      <c r="G136" s="16" t="s">
+      <c r="G136" s="13" t="s">
         <v>568</v>
       </c>
-      <c r="H136" s="15" t="s">
-        <v>560</v>
+      <c r="H136" s="12" t="s">
+        <v>569</v>
       </c>
       <c r="I136" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J136" s="15">
-        <v>1</v>
+      <c r="J136" s="12">
+        <v>4</v>
       </c>
       <c r="K136" s="12">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="L136" s="19" t="s">
-        <v>21</v>
+        <v>114</v>
       </c>
       <c r="M136" s="18">
-        <v>1.18</v>
+        <v>9.3799999999999994E-2</v>
       </c>
       <c r="N136" s="18">
         <f t="shared" si="10"/>
-        <v>3.54</v>
-      </c>
-      <c r="O136" s="15"/>
-    </row>
-    <row r="137" spans="1:15" ht="24.75" thickBot="1">
+        <v>1.1255999999999999</v>
+      </c>
+      <c r="O136" s="12"/>
+    </row>
+    <row r="137" spans="1:15" ht="15.75" thickBot="1">
       <c r="A137" s="5"/>
       <c r="B137" s="10">
-        <f>ROW(B137)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>135</v>
       </c>
-      <c r="C137" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D137" s="12" t="s">
-        <v>569</v>
-      </c>
-      <c r="E137" s="13" t="s">
+      <c r="C137" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D137" s="15" t="s">
         <v>570</v>
       </c>
-      <c r="F137" s="12" t="s">
+      <c r="E137" s="16" t="s">
         <v>571</v>
       </c>
-      <c r="G137" s="13" t="s">
+      <c r="F137" s="15" t="s">
         <v>572</v>
       </c>
-      <c r="H137" s="12" t="s">
+      <c r="G137" s="16" t="s">
         <v>573</v>
+      </c>
+      <c r="H137" s="15" t="s">
+        <v>574</v>
       </c>
       <c r="I137" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J137" s="12">
-        <v>4</v>
+      <c r="J137" s="15">
+        <v>1</v>
       </c>
       <c r="K137" s="12">
         <f t="shared" si="11"/>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L137" s="19" t="s">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="M137" s="18">
-        <v>9.3799999999999994E-2</v>
+        <v>1.51</v>
       </c>
       <c r="N137" s="18">
         <f t="shared" si="10"/>
-        <v>1.1255999999999999</v>
-      </c>
-      <c r="O137" s="12"/>
-    </row>
-    <row r="138" spans="1:15" ht="15.75" thickBot="1">
+        <v>4.53</v>
+      </c>
+      <c r="O137" s="15"/>
+    </row>
+    <row r="138" spans="1:15" ht="24.75" thickBot="1">
       <c r="A138" s="5"/>
       <c r="B138" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B138)-ROW($B$2)</f>
         <v>136</v>
       </c>
-      <c r="C138" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D138" s="15" t="s">
-        <v>574</v>
-      </c>
-      <c r="E138" s="16" t="s">
+      <c r="C138" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D138" s="12" t="s">
         <v>575</v>
       </c>
-      <c r="F138" s="15" t="s">
+      <c r="E138" s="13" t="s">
         <v>576</v>
       </c>
-      <c r="G138" s="16" t="s">
+      <c r="F138" s="12" t="s">
         <v>577</v>
       </c>
-      <c r="H138" s="15" t="s">
+      <c r="G138" s="13" t="s">
         <v>578</v>
+      </c>
+      <c r="H138" s="12" t="s">
+        <v>556</v>
       </c>
       <c r="I138" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J138" s="15">
+      <c r="J138" s="12">
         <v>1</v>
       </c>
       <c r="K138" s="12">
@@ -9272,42 +9263,42 @@
         <v>21</v>
       </c>
       <c r="M138" s="18">
-        <v>1.51</v>
+        <v>1.79</v>
       </c>
       <c r="N138" s="18">
         <f t="shared" si="10"/>
-        <v>4.53</v>
-      </c>
-      <c r="O138" s="15"/>
-    </row>
-    <row r="139" spans="1:15" ht="24.75" thickBot="1">
+        <v>5.37</v>
+      </c>
+      <c r="O138" s="12"/>
+    </row>
+    <row r="139" spans="1:15" ht="15.75" thickBot="1">
       <c r="A139" s="5"/>
       <c r="B139" s="10">
-        <f>ROW(B139)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>137</v>
       </c>
-      <c r="C139" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D139" s="12" t="s">
+      <c r="C139" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D139" s="15" t="s">
         <v>579</v>
       </c>
-      <c r="E139" s="13" t="s">
+      <c r="E139" s="16" t="s">
         <v>580</v>
       </c>
-      <c r="F139" s="12" t="s">
+      <c r="F139" s="15" t="s">
         <v>581</v>
       </c>
-      <c r="G139" s="13" t="s">
+      <c r="G139" s="16" t="s">
         <v>582</v>
       </c>
-      <c r="H139" s="12" t="s">
-        <v>560</v>
+      <c r="H139" s="15" t="s">
+        <v>583</v>
       </c>
       <c r="I139" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J139" s="12">
+      <c r="J139" s="15">
         <v>1</v>
       </c>
       <c r="K139" s="12">
@@ -9318,42 +9309,42 @@
         <v>21</v>
       </c>
       <c r="M139" s="18">
-        <v>1.79</v>
+        <v>2.5253999999999999</v>
       </c>
       <c r="N139" s="18">
         <f t="shared" si="10"/>
-        <v>5.37</v>
-      </c>
-      <c r="O139" s="12"/>
+        <v>7.5762</v>
+      </c>
+      <c r="O139" s="15"/>
     </row>
     <row r="140" spans="1:15" ht="15.75" thickBot="1">
       <c r="A140" s="5"/>
       <c r="B140" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B140)-ROW($B$2)</f>
         <v>138</v>
       </c>
-      <c r="C140" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D140" s="15" t="s">
-        <v>583</v>
-      </c>
-      <c r="E140" s="16" t="s">
+      <c r="C140" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D140" s="12" t="s">
         <v>584</v>
       </c>
-      <c r="F140" s="15" t="s">
+      <c r="E140" s="13" t="s">
         <v>585</v>
       </c>
-      <c r="G140" s="16" t="s">
+      <c r="F140" s="12" t="s">
+        <v>581</v>
+      </c>
+      <c r="G140" s="13" t="s">
         <v>586</v>
       </c>
-      <c r="H140" s="15" t="s">
+      <c r="H140" s="12" t="s">
         <v>587</v>
       </c>
       <c r="I140" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J140" s="15">
+      <c r="J140" s="12">
         <v>1</v>
       </c>
       <c r="K140" s="12">
@@ -9364,42 +9355,42 @@
         <v>21</v>
       </c>
       <c r="M140" s="18">
-        <v>2.5253999999999999</v>
+        <v>5.57</v>
       </c>
       <c r="N140" s="18">
         <f t="shared" si="10"/>
-        <v>7.5762</v>
-      </c>
-      <c r="O140" s="15"/>
-    </row>
-    <row r="141" spans="1:15" ht="15.75" thickBot="1">
+        <v>16.71</v>
+      </c>
+      <c r="O140" s="12"/>
+    </row>
+    <row r="141" spans="1:15" ht="24.75" thickBot="1">
       <c r="A141" s="5"/>
       <c r="B141" s="10">
-        <f>ROW(B141)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>139</v>
       </c>
-      <c r="C141" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D141" s="12" t="s">
+      <c r="C141" s="14" t="s">
         <v>588</v>
       </c>
-      <c r="E141" s="13" t="s">
+      <c r="D141" s="15" t="s">
         <v>589</v>
       </c>
-      <c r="F141" s="12" t="s">
-        <v>585</v>
-      </c>
-      <c r="G141" s="13" t="s">
+      <c r="E141" s="16" t="s">
         <v>590</v>
       </c>
-      <c r="H141" s="12" t="s">
+      <c r="F141" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G141" s="16" t="s">
         <v>591</v>
+      </c>
+      <c r="H141" s="15" t="s">
+        <v>592</v>
       </c>
       <c r="I141" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J141" s="12">
+      <c r="J141" s="15">
         <v>1</v>
       </c>
       <c r="K141" s="12">
@@ -9410,42 +9401,42 @@
         <v>21</v>
       </c>
       <c r="M141" s="18">
-        <v>5.57</v>
+        <v>18.03</v>
       </c>
       <c r="N141" s="18">
         <f t="shared" si="10"/>
-        <v>16.71</v>
-      </c>
-      <c r="O141" s="12"/>
+        <v>54.09</v>
+      </c>
+      <c r="O141" s="15"/>
     </row>
     <row r="142" spans="1:15" ht="24.75" thickBot="1">
       <c r="A142" s="5"/>
       <c r="B142" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B142)-ROW($B$2)</f>
         <v>140</v>
       </c>
-      <c r="C142" s="14" t="s">
-        <v>592</v>
-      </c>
-      <c r="D142" s="15" t="s">
+      <c r="C142" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D142" s="12" t="s">
         <v>593</v>
       </c>
-      <c r="E142" s="16" t="s">
+      <c r="E142" s="13" t="s">
         <v>594</v>
       </c>
       <c r="F142" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="G142" s="16" t="s">
+      <c r="G142" s="13" t="s">
         <v>595</v>
       </c>
-      <c r="H142" s="15" t="s">
-        <v>596</v>
+      <c r="H142" s="12" t="s">
+        <v>556</v>
       </c>
       <c r="I142" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J142" s="15">
+      <c r="J142" s="12">
         <v>1</v>
       </c>
       <c r="K142" s="12">
@@ -9456,134 +9447,134 @@
         <v>21</v>
       </c>
       <c r="M142" s="18">
-        <v>18.03</v>
+        <v>1.06</v>
       </c>
       <c r="N142" s="18">
         <f t="shared" si="10"/>
-        <v>54.09</v>
-      </c>
-      <c r="O142" s="15"/>
+        <v>3.18</v>
+      </c>
+      <c r="O142" s="12"/>
     </row>
     <row r="143" spans="1:15" ht="24.75" thickBot="1">
       <c r="A143" s="5"/>
       <c r="B143" s="10">
-        <f>ROW(B143)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>141</v>
       </c>
-      <c r="C143" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D143" s="12" t="s">
+      <c r="C143" s="14" t="s">
+        <v>596</v>
+      </c>
+      <c r="D143" s="15" t="s">
         <v>597</v>
       </c>
-      <c r="E143" s="13" t="s">
+      <c r="E143" s="16" t="s">
         <v>598</v>
       </c>
       <c r="F143" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="G143" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="G143" s="16" t="s">
         <v>599</v>
       </c>
-      <c r="H143" s="12" t="s">
-        <v>560</v>
+      <c r="H143" s="15" t="s">
+        <v>600</v>
       </c>
       <c r="I143" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J143" s="12">
-        <v>1</v>
+      <c r="J143" s="15">
+        <v>2</v>
       </c>
       <c r="K143" s="12">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L143" s="19" t="s">
-        <v>21</v>
+        <v>114</v>
       </c>
       <c r="M143" s="18">
-        <v>1.06</v>
+        <v>2.3199999999999998E-2</v>
       </c>
       <c r="N143" s="18">
         <f t="shared" si="10"/>
-        <v>3.18</v>
-      </c>
-      <c r="O143" s="12"/>
+        <v>0.13919999999999999</v>
+      </c>
+      <c r="O143" s="15"/>
     </row>
     <row r="144" spans="1:15" ht="24.75" thickBot="1">
       <c r="A144" s="5"/>
       <c r="B144" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B144)-ROW($B$2)</f>
         <v>142</v>
       </c>
-      <c r="C144" s="14" t="s">
-        <v>600</v>
-      </c>
-      <c r="D144" s="15" t="s">
+      <c r="C144" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D144" s="12" t="s">
         <v>601</v>
       </c>
-      <c r="E144" s="16" t="s">
+      <c r="E144" s="13" t="s">
         <v>602</v>
       </c>
       <c r="F144" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="G144" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="G144" s="13" t="s">
         <v>603</v>
       </c>
-      <c r="H144" s="15" t="s">
+      <c r="H144" s="12" t="s">
         <v>604</v>
       </c>
       <c r="I144" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J144" s="15">
-        <v>2</v>
+      <c r="J144" s="12">
+        <v>1</v>
       </c>
       <c r="K144" s="12">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L144" s="19" t="s">
         <v>114</v>
       </c>
       <c r="M144" s="18">
-        <v>2.3199999999999998E-2</v>
+        <v>8.3531999999999993</v>
       </c>
       <c r="N144" s="18">
         <f t="shared" si="10"/>
-        <v>0.13919999999999999</v>
-      </c>
-      <c r="O144" s="15"/>
-    </row>
-    <row r="145" spans="1:15" ht="24.75" thickBot="1">
+        <v>25.059599999999996</v>
+      </c>
+      <c r="O144" s="12"/>
+    </row>
+    <row r="145" spans="1:15" ht="26.25" thickBot="1">
       <c r="A145" s="5"/>
       <c r="B145" s="10">
-        <f>ROW(B145)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>143</v>
       </c>
-      <c r="C145" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D145" s="12" t="s">
+      <c r="C145" s="14" t="s">
         <v>605</v>
       </c>
-      <c r="E145" s="13" t="s">
+      <c r="D145" s="15" t="s">
         <v>606</v>
       </c>
+      <c r="E145" s="16" t="s">
+        <v>607</v>
+      </c>
       <c r="F145" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="G145" s="13" t="s">
-        <v>607</v>
-      </c>
-      <c r="H145" s="12" t="s">
         <v>608</v>
+      </c>
+      <c r="G145" s="16" t="s">
+        <v>609</v>
+      </c>
+      <c r="H145" s="15" t="s">
+        <v>610</v>
       </c>
       <c r="I145" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J145" s="12">
+      <c r="J145" s="15">
         <v>1</v>
       </c>
       <c r="K145" s="12">
@@ -9594,42 +9585,42 @@
         <v>114</v>
       </c>
       <c r="M145" s="18">
-        <v>8.3531999999999993</v>
+        <v>0.63719999999999999</v>
       </c>
       <c r="N145" s="18">
         <f t="shared" si="10"/>
-        <v>25.0596</v>
-      </c>
-      <c r="O145" s="12"/>
-    </row>
-    <row r="146" spans="1:15" ht="26.25" thickBot="1">
+        <v>1.9116</v>
+      </c>
+      <c r="O145" s="15"/>
+    </row>
+    <row r="146" spans="1:15" ht="60.75" thickBot="1">
       <c r="A146" s="5"/>
       <c r="B146" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B146)-ROW($B$2)</f>
         <v>144</v>
       </c>
-      <c r="C146" s="14" t="s">
-        <v>609</v>
-      </c>
-      <c r="D146" s="15" t="s">
-        <v>610</v>
-      </c>
-      <c r="E146" s="16" t="s">
+      <c r="C146" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D146" s="12" t="s">
         <v>611</v>
       </c>
-      <c r="F146" s="15" t="s">
+      <c r="E146" s="13" t="s">
         <v>612</v>
       </c>
-      <c r="G146" s="16" t="s">
+      <c r="F146" s="12" t="s">
         <v>613</v>
       </c>
-      <c r="H146" s="15" t="s">
+      <c r="G146" s="13" t="s">
         <v>614</v>
+      </c>
+      <c r="H146" s="12" t="s">
+        <v>615</v>
       </c>
       <c r="I146" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J146" s="15">
+      <c r="J146" s="12">
         <v>1</v>
       </c>
       <c r="K146" s="12">
@@ -9640,42 +9631,42 @@
         <v>114</v>
       </c>
       <c r="M146" s="18">
-        <v>0.63719999999999999</v>
+        <v>7.8799999999999995E-2</v>
       </c>
       <c r="N146" s="18">
         <f t="shared" si="10"/>
-        <v>1.9116</v>
-      </c>
-      <c r="O146" s="15"/>
-    </row>
-    <row r="147" spans="1:15" ht="60.75" thickBot="1">
+        <v>0.2364</v>
+      </c>
+      <c r="O146" s="12"/>
+    </row>
+    <row r="147" spans="1:15" ht="15.75" thickBot="1">
       <c r="A147" s="5"/>
       <c r="B147" s="10">
-        <f>ROW(B147)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>145</v>
       </c>
-      <c r="C147" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D147" s="12" t="s">
-        <v>615</v>
-      </c>
-      <c r="E147" s="13" t="s">
+      <c r="C147" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D147" s="15" t="s">
         <v>616</v>
       </c>
-      <c r="F147" s="12" t="s">
+      <c r="E147" s="16" t="s">
         <v>617</v>
       </c>
-      <c r="G147" s="13" t="s">
+      <c r="F147" s="15" t="s">
         <v>618</v>
       </c>
-      <c r="H147" s="12" t="s">
+      <c r="G147" s="16" t="s">
         <v>619</v>
+      </c>
+      <c r="H147" s="15" t="s">
+        <v>620</v>
       </c>
       <c r="I147" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J147" s="12">
+      <c r="J147" s="15">
         <v>1</v>
       </c>
       <c r="K147" s="12">
@@ -9683,45 +9674,45 @@
         <v>3</v>
       </c>
       <c r="L147" s="19" t="s">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="M147" s="18">
-        <v>7.8799999999999995E-2</v>
+        <v>4.4400000000000004</v>
       </c>
       <c r="N147" s="18">
         <f t="shared" si="10"/>
-        <v>0.2364</v>
-      </c>
-      <c r="O147" s="12"/>
-    </row>
-    <row r="148" spans="1:15" ht="15.75" thickBot="1">
+        <v>13.32</v>
+      </c>
+      <c r="O147" s="15"/>
+    </row>
+    <row r="148" spans="1:15" ht="24.75" thickBot="1">
       <c r="A148" s="5"/>
       <c r="B148" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B148)-ROW($B$2)</f>
         <v>146</v>
       </c>
-      <c r="C148" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D148" s="15" t="s">
-        <v>620</v>
-      </c>
-      <c r="E148" s="16" t="s">
+      <c r="C148" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D148" s="12" t="s">
         <v>621</v>
       </c>
-      <c r="F148" s="15" t="s">
+      <c r="E148" s="13" t="s">
         <v>622</v>
       </c>
-      <c r="G148" s="16" t="s">
+      <c r="F148" s="12" t="s">
         <v>623</v>
       </c>
-      <c r="H148" s="15" t="s">
+      <c r="G148" s="13" t="s">
         <v>624</v>
+      </c>
+      <c r="H148" s="12" t="s">
+        <v>556</v>
       </c>
       <c r="I148" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J148" s="15">
+      <c r="J148" s="12">
         <v>1</v>
       </c>
       <c r="K148" s="12">
@@ -9732,77 +9723,77 @@
         <v>21</v>
       </c>
       <c r="M148" s="18">
-        <v>4.4400000000000004</v>
+        <v>0.78</v>
       </c>
       <c r="N148" s="18">
         <f t="shared" si="10"/>
-        <v>13.32</v>
-      </c>
-      <c r="O148" s="15"/>
-    </row>
-    <row r="149" spans="1:15" ht="24.75" thickBot="1">
+        <v>2.34</v>
+      </c>
+      <c r="O148" s="12"/>
+    </row>
+    <row r="149" spans="1:15" ht="15.75" thickBot="1">
       <c r="A149" s="5"/>
       <c r="B149" s="10">
-        <f>ROW(B149)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>147</v>
       </c>
-      <c r="C149" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D149" s="12" t="s">
+      <c r="C149" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D149" s="15" t="s">
         <v>625</v>
       </c>
-      <c r="E149" s="13" t="s">
+      <c r="E149" s="16" t="s">
         <v>626</v>
       </c>
-      <c r="F149" s="12" t="s">
+      <c r="F149" s="15" t="s">
         <v>627</v>
       </c>
-      <c r="G149" s="13" t="s">
+      <c r="G149" s="16" t="s">
         <v>628</v>
       </c>
-      <c r="H149" s="12" t="s">
-        <v>560</v>
+      <c r="H149" s="15" t="s">
+        <v>629</v>
       </c>
       <c r="I149" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J149" s="12">
-        <v>1</v>
+      <c r="J149" s="15">
+        <v>2</v>
       </c>
       <c r="K149" s="12">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L149" s="19" t="s">
-        <v>21</v>
+        <v>114</v>
       </c>
       <c r="M149" s="18">
-        <v>0.78</v>
+        <v>0.99080000000000001</v>
       </c>
       <c r="N149" s="18">
         <f t="shared" si="10"/>
-        <v>2.34</v>
-      </c>
-      <c r="O149" s="12"/>
-    </row>
-    <row r="150" spans="1:15" ht="15.75" thickBot="1">
+        <v>5.9447999999999999</v>
+      </c>
+      <c r="O149" s="15"/>
+    </row>
+    <row r="150" spans="1:15" ht="24.75" thickBot="1">
       <c r="A150" s="5"/>
       <c r="B150" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B150)-ROW($B$2)</f>
         <v>148</v>
       </c>
       <c r="C150" s="14" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="D150" s="15" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E150" s="16" t="s">
-        <v>630</v>
-      </c>
-      <c r="F150" s="15" t="s">
         <v>631</v>
+      </c>
+      <c r="F150" s="12" t="s">
+        <v>111</v>
       </c>
       <c r="G150" s="16" t="s">
         <v>632</v>
@@ -9814,47 +9805,47 @@
         <v>150</v>
       </c>
       <c r="J150" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K150" s="12">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L150" s="19" t="s">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="M150" s="18">
-        <v>0.99080000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="N150" s="18">
         <f t="shared" si="10"/>
-        <v>5.9447999999999999</v>
+        <v>1.6800000000000002</v>
       </c>
       <c r="O150" s="15"/>
     </row>
-    <row r="151" spans="1:15" ht="24.75" thickBot="1">
+    <row r="151" spans="1:15" ht="15.75" thickBot="1">
       <c r="A151" s="5"/>
       <c r="B151" s="10">
         <f>ROW(B151)-ROW($B$2)</f>
         <v>149</v>
       </c>
-      <c r="C151" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D151" s="15" t="s">
+      <c r="C151" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D151" s="12" t="s">
         <v>634</v>
       </c>
-      <c r="E151" s="16" t="s">
+      <c r="E151" s="12" t="s">
         <v>635</v>
       </c>
       <c r="F151" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="G151" s="16" t="s">
         <v>636</v>
       </c>
-      <c r="H151" s="15" t="s">
+      <c r="G151" s="12" t="s">
         <v>637</v>
+      </c>
+      <c r="H151" s="12" t="s">
+        <v>638</v>
       </c>
       <c r="I151" s="16" t="s">
         <v>150</v>
@@ -9870,37 +9861,37 @@
         <v>21</v>
       </c>
       <c r="M151" s="18">
-        <v>0.56000000000000005</v>
+        <v>2.89</v>
       </c>
       <c r="N151" s="18">
         <f t="shared" si="10"/>
-        <v>1.68</v>
+        <v>8.67</v>
       </c>
       <c r="O151" s="15"/>
     </row>
-    <row r="152" spans="1:15" ht="15.75" thickBot="1">
+    <row r="152" spans="1:15" ht="24.75" thickBot="1">
       <c r="A152" s="5"/>
       <c r="B152" s="10">
-        <f>ROW(B152)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>150</v>
       </c>
-      <c r="C152" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D152" s="12" t="s">
-        <v>638</v>
-      </c>
-      <c r="E152" s="12" t="s">
+      <c r="C152" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D152" s="15" t="s">
         <v>639</v>
       </c>
-      <c r="F152" s="12" t="s">
+      <c r="E152" s="16" t="s">
         <v>640</v>
       </c>
-      <c r="G152" s="12" t="s">
+      <c r="F152" s="15" t="s">
         <v>641</v>
       </c>
-      <c r="H152" s="12" t="s">
+      <c r="G152" s="16" t="s">
         <v>642</v>
+      </c>
+      <c r="H152" s="15" t="s">
+        <v>643</v>
       </c>
       <c r="I152" s="16" t="s">
         <v>150</v>
@@ -9916,42 +9907,42 @@
         <v>21</v>
       </c>
       <c r="M152" s="18">
-        <v>2.89</v>
+        <v>1.35</v>
       </c>
       <c r="N152" s="18">
         <f t="shared" si="10"/>
-        <v>8.67</v>
+        <v>4.0500000000000007</v>
       </c>
       <c r="O152" s="15"/>
     </row>
     <row r="153" spans="1:15" ht="24.75" thickBot="1">
       <c r="A153" s="5"/>
       <c r="B153" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B153)-ROW($B$2)</f>
         <v>151</v>
       </c>
-      <c r="C153" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D153" s="15" t="s">
-        <v>643</v>
-      </c>
-      <c r="E153" s="16" t="s">
+      <c r="C153" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D153" s="12" t="s">
         <v>644</v>
       </c>
-      <c r="F153" s="15" t="s">
+      <c r="E153" s="13" t="s">
         <v>645</v>
       </c>
-      <c r="G153" s="16" t="s">
+      <c r="F153" s="12" t="s">
         <v>646</v>
       </c>
-      <c r="H153" s="15" t="s">
+      <c r="G153" s="13" t="s">
         <v>647</v>
+      </c>
+      <c r="H153" s="12" t="s">
+        <v>556</v>
       </c>
       <c r="I153" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J153" s="15">
+      <c r="J153" s="12">
         <v>1</v>
       </c>
       <c r="K153" s="12">
@@ -9962,42 +9953,42 @@
         <v>21</v>
       </c>
       <c r="M153" s="18">
-        <v>1.35</v>
+        <v>2.13</v>
       </c>
       <c r="N153" s="18">
         <f t="shared" si="10"/>
-        <v>4.05</v>
-      </c>
-      <c r="O153" s="15"/>
-    </row>
-    <row r="154" spans="1:15" ht="24.75" thickBot="1">
+        <v>6.39</v>
+      </c>
+      <c r="O153" s="12"/>
+    </row>
+    <row r="154" spans="1:15" ht="15.75" thickBot="1">
       <c r="A154" s="5"/>
       <c r="B154" s="10">
-        <f>ROW(B154)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>152</v>
       </c>
-      <c r="C154" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D154" s="12" t="s">
+      <c r="C154" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D154" s="15" t="s">
         <v>648</v>
       </c>
-      <c r="E154" s="13" t="s">
+      <c r="E154" s="16" t="s">
         <v>649</v>
       </c>
-      <c r="F154" s="12" t="s">
+      <c r="F154" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G154" s="16" t="s">
         <v>650</v>
       </c>
-      <c r="G154" s="13" t="s">
+      <c r="H154" s="15" t="s">
         <v>651</v>
-      </c>
-      <c r="H154" s="12" t="s">
-        <v>560</v>
       </c>
       <c r="I154" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J154" s="12">
+      <c r="J154" s="15">
         <v>1</v>
       </c>
       <c r="K154" s="12">
@@ -10008,42 +9999,42 @@
         <v>21</v>
       </c>
       <c r="M154" s="18">
-        <v>2.13</v>
+        <v>0.15684999999999999</v>
       </c>
       <c r="N154" s="18">
         <f t="shared" si="10"/>
-        <v>6.39</v>
-      </c>
-      <c r="O154" s="12"/>
+        <v>0.47054999999999997</v>
+      </c>
+      <c r="O154" s="15"/>
     </row>
     <row r="155" spans="1:15" ht="15.75" thickBot="1">
       <c r="A155" s="5"/>
       <c r="B155" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B155)-ROW($B$2)</f>
         <v>153</v>
       </c>
-      <c r="C155" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D155" s="15" t="s">
+      <c r="C155" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D155" s="12" t="s">
         <v>652</v>
       </c>
-      <c r="E155" s="16" t="s">
+      <c r="E155" s="13" t="s">
         <v>653</v>
       </c>
-      <c r="F155" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="G155" s="16" t="s">
+      <c r="F155" s="12" t="s">
         <v>654</v>
       </c>
-      <c r="H155" s="15" t="s">
+      <c r="G155" s="13" t="s">
         <v>655</v>
+      </c>
+      <c r="H155" s="12" t="s">
+        <v>656</v>
       </c>
       <c r="I155" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J155" s="15">
+      <c r="J155" s="12">
         <v>1</v>
       </c>
       <c r="K155" s="12">
@@ -10054,42 +10045,42 @@
         <v>21</v>
       </c>
       <c r="M155" s="18">
-        <v>0.15684999999999999</v>
+        <v>0.36</v>
       </c>
       <c r="N155" s="18">
         <f t="shared" si="10"/>
-        <v>0.47055000000000002</v>
-      </c>
-      <c r="O155" s="15"/>
-    </row>
-    <row r="156" spans="1:15" ht="15.75" thickBot="1">
+        <v>1.08</v>
+      </c>
+      <c r="O155" s="12"/>
+    </row>
+    <row r="156" spans="1:15" ht="24.75" thickBot="1">
       <c r="A156" s="5"/>
       <c r="B156" s="10">
-        <f>ROW(B156)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>154</v>
       </c>
-      <c r="C156" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D156" s="12" t="s">
-        <v>656</v>
-      </c>
-      <c r="E156" s="13" t="s">
+      <c r="C156" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D156" s="15" t="s">
         <v>657</v>
       </c>
-      <c r="F156" s="12" t="s">
+      <c r="E156" s="16" t="s">
         <v>658</v>
       </c>
-      <c r="G156" s="13" t="s">
+      <c r="F156" s="15" t="s">
         <v>659</v>
       </c>
-      <c r="H156" s="12" t="s">
+      <c r="G156" s="16" t="s">
         <v>660</v>
+      </c>
+      <c r="H156" s="15" t="s">
+        <v>661</v>
       </c>
       <c r="I156" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J156" s="12">
+      <c r="J156" s="15">
         <v>1</v>
       </c>
       <c r="K156" s="12">
@@ -10097,45 +10088,45 @@
         <v>3</v>
       </c>
       <c r="L156" s="19" t="s">
-        <v>21</v>
+        <v>114</v>
       </c>
       <c r="M156" s="18">
-        <v>0.36</v>
+        <v>0.34460000000000002</v>
       </c>
       <c r="N156" s="18">
         <f t="shared" si="10"/>
-        <v>1.08</v>
-      </c>
-      <c r="O156" s="12"/>
-    </row>
-    <row r="157" spans="1:15" ht="24.75" thickBot="1">
+        <v>1.0338000000000001</v>
+      </c>
+      <c r="O156" s="15"/>
+    </row>
+    <row r="157" spans="1:15" ht="36.75" thickBot="1">
       <c r="A157" s="5"/>
       <c r="B157" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B157)-ROW($B$2)</f>
         <v>155</v>
       </c>
-      <c r="C157" s="14" t="s">
-        <v>552</v>
-      </c>
-      <c r="D157" s="15" t="s">
-        <v>661</v>
-      </c>
-      <c r="E157" s="16" t="s">
+      <c r="C157" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="D157" s="12" t="s">
         <v>662</v>
       </c>
-      <c r="F157" s="15" t="s">
+      <c r="E157" s="13" t="s">
         <v>663</v>
       </c>
-      <c r="G157" s="16" t="s">
+      <c r="F157" s="12" t="s">
         <v>664</v>
       </c>
-      <c r="H157" s="15" t="s">
+      <c r="G157" s="13" t="s">
         <v>665</v>
+      </c>
+      <c r="H157" s="12" t="s">
+        <v>666</v>
       </c>
       <c r="I157" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="J157" s="15">
+      <c r="J157" s="12">
         <v>1</v>
       </c>
       <c r="K157" s="12">
@@ -10143,45 +10134,45 @@
         <v>3</v>
       </c>
       <c r="L157" s="19" t="s">
-        <v>114</v>
+        <v>21</v>
       </c>
       <c r="M157" s="18">
-        <v>0.34460000000000002</v>
+        <v>0.94</v>
       </c>
       <c r="N157" s="18">
         <f t="shared" si="10"/>
-        <v>1.0338000000000001</v>
-      </c>
-      <c r="O157" s="15"/>
+        <v>2.82</v>
+      </c>
+      <c r="O157" s="12"/>
     </row>
     <row r="158" spans="1:15" ht="36.75" thickBot="1">
       <c r="A158" s="5"/>
       <c r="B158" s="10">
-        <f>ROW(B158)-ROW($B$2)</f>
+        <f t="shared" si="8"/>
         <v>156</v>
       </c>
-      <c r="C158" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="D158" s="12" t="s">
-        <v>666</v>
-      </c>
-      <c r="E158" s="13" t="s">
+      <c r="C158" s="14" t="s">
         <v>667</v>
       </c>
-      <c r="F158" s="12" t="s">
+      <c r="D158" s="15" t="s">
         <v>668</v>
       </c>
-      <c r="G158" s="13" t="s">
+      <c r="E158" s="16" t="s">
         <v>669</v>
       </c>
-      <c r="H158" s="12" t="s">
+      <c r="F158" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G158" s="16" t="s">
         <v>670</v>
       </c>
+      <c r="H158" s="15" t="s">
+        <v>671</v>
+      </c>
       <c r="I158" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="J158" s="12">
+        <v>672</v>
+      </c>
+      <c r="J158" s="15">
         <v>1</v>
       </c>
       <c r="K158" s="12">
@@ -10192,171 +10183,169 @@
         <v>21</v>
       </c>
       <c r="M158" s="18">
-        <v>0.94</v>
+        <v>0.28784999999999999</v>
       </c>
       <c r="N158" s="18">
         <f t="shared" si="10"/>
-        <v>2.82</v>
-      </c>
-      <c r="O158" s="12"/>
-    </row>
-    <row r="159" spans="1:15" ht="36.75" thickBot="1">
+        <v>0.86355000000000004</v>
+      </c>
+      <c r="O158" s="15"/>
+    </row>
+    <row r="159" spans="1:15" ht="15.75" thickBot="1">
       <c r="A159" s="5"/>
       <c r="B159" s="10">
-        <f t="shared" si="8"/>
+        <f>ROW(B159)-ROW($B$2)</f>
         <v>157</v>
       </c>
-      <c r="C159" s="14" t="s">
-        <v>671</v>
-      </c>
-      <c r="D159" s="15" t="s">
-        <v>672</v>
-      </c>
-      <c r="E159" s="16" t="s">
+      <c r="C159" s="11" t="s">
+        <v>667</v>
+      </c>
+      <c r="D159" s="12" t="s">
         <v>673</v>
+      </c>
+      <c r="E159" s="13" t="s">
+        <v>674</v>
       </c>
       <c r="F159" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="G159" s="16" t="s">
-        <v>674</v>
-      </c>
-      <c r="H159" s="15" t="s">
+      <c r="G159" s="13" t="s">
         <v>675</v>
       </c>
-      <c r="I159" s="16" t="s">
+      <c r="H159" s="12" t="s">
         <v>676</v>
       </c>
-      <c r="J159" s="15">
-        <v>1</v>
+      <c r="I159" s="13" t="s">
+        <v>677</v>
+      </c>
+      <c r="J159" s="12">
+        <v>2</v>
       </c>
       <c r="K159" s="12">
         <f t="shared" si="11"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L159" s="19" t="s">
         <v>21</v>
       </c>
       <c r="M159" s="18">
-        <v>0.28784999999999999</v>
+        <v>0.80600000000000005</v>
       </c>
       <c r="N159" s="18">
         <f t="shared" si="10"/>
-        <v>0.86355000000000004</v>
-      </c>
-      <c r="O159" s="15"/>
-    </row>
-    <row r="160" spans="1:15" ht="15.75" thickBot="1">
-      <c r="A160" s="5"/>
+        <v>4.8360000000000003</v>
+      </c>
+      <c r="O159" s="12"/>
+    </row>
+    <row r="160" spans="1:15" ht="24.75" thickBot="1">
       <c r="B160" s="10">
-        <f>ROW(B160)-ROW($B$2)</f>
+        <f t="shared" ref="B160:B166" si="12">ROW(B160)-ROW($B$2)</f>
         <v>158</v>
       </c>
       <c r="C160" s="11" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
       <c r="D160" s="12" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="E160" s="13" t="s">
-        <v>678</v>
+        <v>712</v>
       </c>
       <c r="F160" s="15" t="s">
         <v>111</v>
       </c>
       <c r="G160" s="13" t="s">
-        <v>679</v>
+        <v>713</v>
       </c>
       <c r="H160" s="12" t="s">
-        <v>680</v>
-      </c>
-      <c r="I160" s="13" t="s">
-        <v>681</v>
-      </c>
+        <v>249</v>
+      </c>
+      <c r="I160" s="13"/>
       <c r="J160" s="12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K160" s="12">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L160" s="19" t="s">
-        <v>21</v>
+        <v>114</v>
       </c>
       <c r="M160" s="18">
-        <v>0.80600000000000005</v>
+        <v>1.0093000000000001</v>
       </c>
       <c r="N160" s="18">
-        <f t="shared" si="10"/>
-        <v>4.8360000000000003</v>
+        <f>M160*K160</f>
+        <v>3.0279000000000003</v>
       </c>
       <c r="O160" s="12"/>
     </row>
-    <row r="161" spans="2:19" ht="24.75" thickBot="1">
+    <row r="161" spans="2:19" ht="36.75" thickBot="1">
       <c r="B161" s="10">
-        <f t="shared" ref="B161:B167" si="12">ROW(B161)-ROW($B$2)</f>
+        <f t="shared" si="12"/>
         <v>159</v>
       </c>
       <c r="C161" s="11" t="s">
+        <v>678</v>
+      </c>
+      <c r="D161" s="12" t="s">
+        <v>680</v>
+      </c>
+      <c r="E161" s="13" t="s">
+        <v>681</v>
+      </c>
+      <c r="F161" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="G161" s="13" t="s">
         <v>682</v>
-      </c>
-      <c r="D161" s="12" t="s">
-        <v>683</v>
-      </c>
-      <c r="E161" s="13" t="s">
-        <v>716</v>
-      </c>
-      <c r="F161" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="G161" s="13" t="s">
-        <v>717</v>
       </c>
       <c r="H161" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="I161" s="13"/>
+      <c r="I161" s="13" t="s">
+        <v>150</v>
+      </c>
       <c r="J161" s="12">
         <v>1</v>
       </c>
       <c r="K161" s="12">
-        <f t="shared" si="11"/>
         <v>3</v>
       </c>
-      <c r="L161" s="19" t="s">
+      <c r="L161" s="17" t="s">
         <v>114</v>
       </c>
       <c r="M161" s="18">
-        <v>1.0093000000000001</v>
+        <v>0.43</v>
       </c>
       <c r="N161" s="18">
         <f>M161*K161</f>
-        <v>3.0279000000000003</v>
+        <v>1.29</v>
       </c>
       <c r="O161" s="12"/>
     </row>
-    <row r="162" spans="2:19" ht="36.75" thickBot="1">
+    <row r="162" spans="2:19" ht="30.75" thickBot="1">
       <c r="B162" s="10">
         <f t="shared" si="12"/>
         <v>160</v>
       </c>
       <c r="C162" s="11" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="D162" s="12" t="s">
+        <v>683</v>
+      </c>
+      <c r="E162" s="13" t="s">
         <v>684</v>
-      </c>
-      <c r="E162" s="13" t="s">
-        <v>685</v>
       </c>
       <c r="F162" s="15" t="s">
         <v>150</v>
       </c>
       <c r="G162" s="13" t="s">
-        <v>686</v>
+        <v>150</v>
       </c>
       <c r="H162" s="12" t="s">
-        <v>249</v>
+        <v>685</v>
       </c>
       <c r="I162" s="13" t="s">
         <v>150</v>
@@ -10367,25 +10356,25 @@
       <c r="K162" s="12">
         <v>3</v>
       </c>
-      <c r="L162" s="17" t="s">
-        <v>114</v>
+      <c r="L162" s="19" t="s">
+        <v>686</v>
       </c>
       <c r="M162" s="18">
-        <v>0.43</v>
+        <v>9.8699999999999992</v>
       </c>
       <c r="N162" s="18">
         <f>M162*K162</f>
-        <v>1.29</v>
+        <v>29.61</v>
       </c>
       <c r="O162" s="12"/>
     </row>
-    <row r="163" spans="2:19" ht="30.75" thickBot="1">
+    <row r="163" spans="2:19" ht="15.75" thickBot="1">
       <c r="B163" s="10">
         <f t="shared" si="12"/>
         <v>161</v>
       </c>
       <c r="C163" s="11" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="D163" s="12" t="s">
         <v>687</v>
@@ -10397,10 +10386,10 @@
         <v>150</v>
       </c>
       <c r="G163" s="13" t="s">
-        <v>150</v>
+        <v>689</v>
       </c>
       <c r="H163" s="12" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="I163" s="13" t="s">
         <v>150</v>
@@ -10412,59 +10401,46 @@
         <v>3</v>
       </c>
       <c r="L163" s="19" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="M163" s="18">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="N163" s="18">
         <f>M163*K163</f>
-        <v>21</v>
+        <v>297</v>
       </c>
       <c r="O163" s="12"/>
     </row>
-    <row r="164" spans="2:19" ht="15.75" thickBot="1">
+    <row r="164" spans="2:19" ht="24.75" thickBot="1">
       <c r="B164" s="10">
         <f t="shared" si="12"/>
         <v>162</v>
       </c>
       <c r="C164" s="11" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="D164" s="12" t="s">
-        <v>691</v>
+        <v>150</v>
       </c>
       <c r="E164" s="13" t="s">
         <v>692</v>
       </c>
-      <c r="F164" s="15" t="s">
-        <v>150</v>
-      </c>
+      <c r="F164" s="15"/>
       <c r="G164" s="13" t="s">
         <v>693</v>
       </c>
       <c r="H164" s="12" t="s">
         <v>694</v>
       </c>
-      <c r="I164" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="J164" s="12">
-        <v>1</v>
-      </c>
-      <c r="K164" s="12">
-        <v>3</v>
-      </c>
-      <c r="L164" s="19" t="s">
-        <v>695</v>
-      </c>
-      <c r="M164" s="18">
-        <v>99</v>
-      </c>
-      <c r="N164" s="18">
-        <f>M164*K164</f>
-        <v>297</v>
-      </c>
+      <c r="I164" s="13"/>
+      <c r="J164" s="12"/>
+      <c r="K164" s="12"/>
+      <c r="L164" s="17" t="s">
+        <v>694</v>
+      </c>
+      <c r="M164" s="18"/>
+      <c r="N164" s="18"/>
       <c r="O164" s="12"/>
     </row>
     <row r="165" spans="2:19" ht="24.75" thickBot="1">
@@ -10473,51 +10449,51 @@
         <v>163</v>
       </c>
       <c r="C165" s="11" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="D165" s="12" t="s">
         <v>150</v>
       </c>
       <c r="E165" s="13" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="F165" s="15"/>
       <c r="G165" s="13" t="s">
+        <v>696</v>
+      </c>
+      <c r="H165" s="12" t="s">
         <v>697</v>
-      </c>
-      <c r="H165" s="12" t="s">
-        <v>698</v>
       </c>
       <c r="I165" s="13"/>
       <c r="J165" s="12"/>
       <c r="K165" s="12"/>
       <c r="L165" s="17" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="M165" s="18"/>
       <c r="N165" s="18"/>
       <c r="O165" s="12"/>
     </row>
-    <row r="166" spans="2:19" ht="24.75" thickBot="1">
+    <row r="166" spans="2:19" s="3" customFormat="1" ht="24.75" thickBot="1">
       <c r="B166" s="10">
         <f t="shared" si="12"/>
         <v>164</v>
       </c>
       <c r="C166" s="11" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="D166" s="12" t="s">
         <v>150</v>
       </c>
       <c r="E166" s="13" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="F166" s="15"/>
       <c r="G166" s="13" t="s">
+        <v>699</v>
+      </c>
+      <c r="H166" s="12" t="s">
         <v>700</v>
-      </c>
-      <c r="H166" s="12" t="s">
-        <v>701</v>
       </c>
       <c r="I166" s="13"/>
       <c r="J166" s="12"/>
@@ -10525,60 +10501,29 @@
       <c r="L166" s="17" t="s">
         <v>701</v>
       </c>
-      <c r="M166" s="18"/>
-      <c r="N166" s="18"/>
+      <c r="M166" s="41"/>
+      <c r="N166" s="41"/>
       <c r="O166" s="12"/>
-    </row>
-    <row r="167" spans="2:19" s="3" customFormat="1" ht="24.75" thickBot="1">
-      <c r="B167" s="10">
-        <f t="shared" si="12"/>
-        <v>165</v>
-      </c>
-      <c r="C167" s="11" t="s">
-        <v>682</v>
-      </c>
-      <c r="D167" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="E167" s="13" t="s">
+      <c r="Q166"/>
+      <c r="R166"/>
+      <c r="S166"/>
+    </row>
+    <row r="167" spans="2:19">
+      <c r="M167" s="42" t="s">
         <v>702</v>
       </c>
-      <c r="F167" s="15"/>
-      <c r="G167" s="13" t="s">
+      <c r="N167" s="43">
+        <f>SUM(N3:N166)</f>
+        <v>779.40039000000013</v>
+      </c>
+    </row>
+    <row r="168" spans="2:19" ht="15.75" thickBot="1">
+      <c r="M168" s="44" t="s">
         <v>703</v>
       </c>
-      <c r="H167" s="12" t="s">
-        <v>704</v>
-      </c>
-      <c r="I167" s="13"/>
-      <c r="J167" s="12"/>
-      <c r="K167" s="12"/>
-      <c r="L167" s="17" t="s">
-        <v>705</v>
-      </c>
-      <c r="M167" s="41"/>
-      <c r="N167" s="41"/>
-      <c r="O167" s="12"/>
-      <c r="Q167"/>
-      <c r="R167"/>
-      <c r="S167"/>
-    </row>
-    <row r="168" spans="2:19">
-      <c r="M168" s="42" t="s">
-        <v>706</v>
-      </c>
-      <c r="N168" s="43">
-        <f>SUM(N3:N167)</f>
-        <v>770.82039000000009</v>
-      </c>
-    </row>
-    <row r="169" spans="2:19" ht="15.75" thickBot="1">
-      <c r="M169" s="44" t="s">
-        <v>707</v>
-      </c>
-      <c r="N169" s="45">
-        <f>N168/3</f>
-        <v>256.94013000000001</v>
+      <c r="N168" s="45">
+        <f>N167/3</f>
+        <v>259.80013000000002</v>
       </c>
     </row>
   </sheetData>
@@ -10710,7 +10655,7 @@
     <hyperlink ref="L130" r:id="rId122"/>
     <hyperlink ref="L131" r:id="rId123"/>
     <hyperlink ref="L132" r:id="rId124"/>
-    <hyperlink ref="L133" r:id="rId125"/>
+    <hyperlink ref="L134" r:id="rId125"/>
     <hyperlink ref="L135" r:id="rId126"/>
     <hyperlink ref="L136" r:id="rId127"/>
     <hyperlink ref="L137" r:id="rId128"/>
@@ -10736,16 +10681,15 @@
     <hyperlink ref="L157" r:id="rId148"/>
     <hyperlink ref="L158" r:id="rId149"/>
     <hyperlink ref="L159" r:id="rId150"/>
-    <hyperlink ref="L160" r:id="rId151"/>
-    <hyperlink ref="L166" r:id="rId152"/>
-    <hyperlink ref="L165" r:id="rId153"/>
-    <hyperlink ref="L167" r:id="rId154"/>
-    <hyperlink ref="L163" r:id="rId155"/>
-    <hyperlink ref="L162" r:id="rId156"/>
-    <hyperlink ref="L56" r:id="rId157"/>
-    <hyperlink ref="L71" r:id="rId158"/>
-    <hyperlink ref="L134" r:id="rId159"/>
-    <hyperlink ref="L161" r:id="rId160"/>
+    <hyperlink ref="L165" r:id="rId151"/>
+    <hyperlink ref="L164" r:id="rId152"/>
+    <hyperlink ref="L166" r:id="rId153"/>
+    <hyperlink ref="L162" r:id="rId154"/>
+    <hyperlink ref="L161" r:id="rId155"/>
+    <hyperlink ref="L56" r:id="rId156"/>
+    <hyperlink ref="L71" r:id="rId157"/>
+    <hyperlink ref="L133" r:id="rId158"/>
+    <hyperlink ref="L160" r:id="rId159"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
#4 Chock Part no update in BOM.
</commit_message>
<xml_diff>
--- a/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
+++ b/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
@@ -2150,9 +2150,6 @@
     <t>HJ-SMA175</t>
   </si>
   <si>
-    <t>MCZ1210CH900CPTA0G</t>
-  </si>
-  <si>
     <t>MAX3232EIDR</t>
   </si>
   <si>
@@ -2178,6 +2175,9 @@
   </si>
   <si>
     <t>R58, R66, R98</t>
+  </si>
+  <si>
+    <t>MCZ1210CH900L2TA0G</t>
   </si>
 </sst>
 </file>
@@ -5441,13 +5441,13 @@
         <v>54</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="D56" s="15" t="s">
         <v>248</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F56" s="15" t="s">
         <v>111</v>
@@ -5456,7 +5456,7 @@
         <v>704</v>
       </c>
       <c r="H56" s="15" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="I56" s="16" t="s">
         <v>150</v>
@@ -6131,7 +6131,7 @@
         <v>69</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="D71" s="15" t="s">
         <v>307</v>
@@ -6143,7 +6143,7 @@
         <v>111</v>
       </c>
       <c r="G71" s="15" t="s">
-        <v>705</v>
+        <v>714</v>
       </c>
       <c r="H71" s="15" t="s">
         <v>53</v>
@@ -7844,7 +7844,7 @@
         <v>386</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="E108" s="16" t="s">
         <v>462</v>
@@ -9008,13 +9008,13 @@
         <v>554</v>
       </c>
       <c r="E133" s="12" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="F133" s="12" t="s">
         <v>555</v>
       </c>
       <c r="G133" s="12" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H133" s="12" t="s">
         <v>556</v>
@@ -10249,13 +10249,13 @@
         <v>679</v>
       </c>
       <c r="E160" s="13" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="F160" s="15" t="s">
         <v>111</v>
       </c>
       <c r="G160" s="13" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="H160" s="12" t="s">
         <v>249</v>

</xml_diff>

<commit_message>
#4 Client and eSpark BOM Peripheral added
</commit_message>
<xml_diff>
--- a/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
+++ b/Design-Files/Carrier-Board-v1.0/BOM/Client BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1376" uniqueCount="725">
   <si>
     <t>#</t>
   </si>
@@ -2171,6 +2171,30 @@
   </si>
   <si>
     <t>Surge Protection (TVS/ESD)</t>
+  </si>
+  <si>
+    <t>250V 10A 3 -40℃~+105℃ 1.5 1 16~28 3.5mm 1x3P Green Plug P=3.5mm Pluggable System Terminal Block ROHS</t>
+  </si>
+  <si>
+    <t>DB2EK-3.5-3P-GN-S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DORABO </t>
+  </si>
+  <si>
+    <t>Network cables ROHS</t>
+  </si>
+  <si>
+    <t>S108510003</t>
+  </si>
+  <si>
+    <t>Ckmtw</t>
+  </si>
+  <si>
+    <t>S108510001</t>
+  </si>
+  <si>
+    <t>S108510002</t>
   </si>
 </sst>
 </file>
@@ -2496,7 +2520,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -2623,6 +2647,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2907,7 +2934,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:V170"/>
+  <dimension ref="A1:V174"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="4.5703125" style="4" customWidth="1"/>
@@ -8444,7 +8471,7 @@
         <v>0.1</v>
       </c>
       <c r="N120" s="18">
-        <f t="shared" ref="N120:N159" si="11">M120*K120</f>
+        <f t="shared" ref="N120:N163" si="11">M120*K120</f>
         <v>0.60000000000000009</v>
       </c>
       <c r="O120" s="15"/>
@@ -8947,7 +8974,7 @@
         <v>6</v>
       </c>
       <c r="K131" s="12">
-        <f t="shared" ref="K131:K160" si="12">3*J131</f>
+        <f t="shared" ref="K131:K164" si="12">3*J131</f>
         <v>18</v>
       </c>
       <c r="L131" s="19" t="s">
@@ -10250,118 +10277,121 @@
       </c>
       <c r="O159" s="12"/>
     </row>
-    <row r="160" spans="1:15" ht="24.75" thickBot="1">
+    <row r="160" spans="1:15" ht="15.75" thickBot="1">
       <c r="A160" s="5"/>
       <c r="B160" s="10">
-        <f t="shared" ref="B160:B167" si="13">ROW(B160)-ROW($B$2)</f>
+        <f t="shared" ref="B160:B162" si="13">ROW(B160)-ROW($B$2)</f>
         <v>158</v>
       </c>
-      <c r="C160" s="11" t="s">
+      <c r="C160" s="47" t="s">
         <v>661</v>
       </c>
       <c r="D160" s="12" t="s">
-        <v>662</v>
+        <v>144</v>
       </c>
       <c r="E160" s="13" t="s">
-        <v>694</v>
+        <v>720</v>
       </c>
       <c r="F160" s="15" t="s">
         <v>107</v>
       </c>
       <c r="G160" s="13" t="s">
-        <v>695</v>
+        <v>721</v>
       </c>
       <c r="H160" s="12" t="s">
-        <v>242</v>
-      </c>
-      <c r="I160" s="13"/>
+        <v>722</v>
+      </c>
+      <c r="I160" s="13" t="s">
+        <v>144</v>
+      </c>
       <c r="J160" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K160" s="12">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L160" s="19" t="s">
         <v>110</v>
       </c>
       <c r="M160" s="18">
-        <v>1.0093000000000001</v>
+        <v>0.1767</v>
       </c>
       <c r="N160" s="18">
-        <f>M160*K160</f>
-        <v>3.0279000000000003</v>
+        <f t="shared" si="11"/>
+        <v>1.0602</v>
       </c>
       <c r="O160" s="12"/>
     </row>
-    <row r="161" spans="1:22" ht="36.75" thickBot="1">
+    <row r="161" spans="1:22" ht="15.75" thickBot="1">
       <c r="A161" s="5"/>
       <c r="B161" s="10">
         <f t="shared" si="13"/>
         <v>159</v>
       </c>
-      <c r="C161" s="11" t="s">
+      <c r="C161" s="47" t="s">
         <v>661</v>
       </c>
       <c r="D161" s="12" t="s">
-        <v>663</v>
+        <v>144</v>
       </c>
       <c r="E161" s="13" t="s">
-        <v>664</v>
+        <v>720</v>
       </c>
       <c r="F161" s="15" t="s">
-        <v>144</v>
+        <v>107</v>
       </c>
       <c r="G161" s="13" t="s">
-        <v>665</v>
+        <v>723</v>
       </c>
       <c r="H161" s="12" t="s">
-        <v>242</v>
+        <v>722</v>
       </c>
       <c r="I161" s="13" t="s">
         <v>144</v>
       </c>
       <c r="J161" s="12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K161" s="12">
-        <v>3</v>
-      </c>
-      <c r="L161" s="17" t="s">
+        <f t="shared" si="12"/>
+        <v>9</v>
+      </c>
+      <c r="L161" s="19" t="s">
         <v>110</v>
       </c>
       <c r="M161" s="18">
-        <v>0.43</v>
+        <v>9.1499999999999998E-2</v>
       </c>
       <c r="N161" s="18">
-        <f>M161*K161</f>
-        <v>1.29</v>
+        <f t="shared" si="11"/>
+        <v>0.82350000000000001</v>
       </c>
       <c r="O161" s="12"/>
     </row>
-    <row r="162" spans="1:22" ht="30.75" thickBot="1">
+    <row r="162" spans="1:22" ht="15.75" thickBot="1">
       <c r="A162" s="5"/>
       <c r="B162" s="10">
         <f t="shared" si="13"/>
         <v>160</v>
       </c>
-      <c r="C162" s="11" t="s">
+      <c r="C162" s="47" t="s">
         <v>661</v>
       </c>
       <c r="D162" s="12" t="s">
-        <v>666</v>
+        <v>144</v>
       </c>
       <c r="E162" s="13" t="s">
-        <v>667</v>
+        <v>720</v>
       </c>
       <c r="F162" s="15" t="s">
-        <v>144</v>
+        <v>107</v>
       </c>
       <c r="G162" s="13" t="s">
-        <v>144</v>
+        <v>724</v>
       </c>
       <c r="H162" s="12" t="s">
-        <v>668</v>
+        <v>722</v>
       </c>
       <c r="I162" s="13" t="s">
         <v>144</v>
@@ -10370,252 +10400,433 @@
         <v>1</v>
       </c>
       <c r="K162" s="12">
+        <f t="shared" si="12"/>
         <v>3</v>
       </c>
       <c r="L162" s="19" t="s">
-        <v>669</v>
+        <v>110</v>
       </c>
       <c r="M162" s="18">
-        <v>9.8699999999999992</v>
+        <v>0.1381</v>
       </c>
       <c r="N162" s="18">
-        <f>M162*K162</f>
-        <v>29.61</v>
+        <f t="shared" si="11"/>
+        <v>0.4143</v>
       </c>
       <c r="O162" s="12"/>
     </row>
-    <row r="163" spans="1:22" ht="15.75" thickBot="1">
+    <row r="163" spans="1:22" ht="48.75" thickBot="1">
+      <c r="A163" s="5"/>
       <c r="B163" s="10">
-        <f t="shared" si="13"/>
+        <f>ROW(B163)-ROW($B$2)</f>
         <v>161</v>
       </c>
-      <c r="C163" s="11" t="s">
+      <c r="C163" s="47" t="s">
         <v>661</v>
       </c>
       <c r="D163" s="12" t="s">
-        <v>670</v>
+        <v>144</v>
       </c>
       <c r="E163" s="13" t="s">
-        <v>671</v>
+        <v>717</v>
       </c>
       <c r="F163" s="15" t="s">
-        <v>144</v>
+        <v>107</v>
       </c>
       <c r="G163" s="13" t="s">
-        <v>672</v>
+        <v>718</v>
       </c>
       <c r="H163" s="12" t="s">
-        <v>673</v>
+        <v>719</v>
       </c>
       <c r="I163" s="13" t="s">
         <v>144</v>
       </c>
       <c r="J163" s="12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K163" s="12">
-        <v>3</v>
+        <f t="shared" si="12"/>
+        <v>15</v>
       </c>
       <c r="L163" s="19" t="s">
-        <v>674</v>
+        <v>110</v>
       </c>
       <c r="M163" s="18">
-        <v>99</v>
+        <v>0.28139999999999998</v>
       </c>
       <c r="N163" s="18">
-        <f>M163*K163</f>
-        <v>297</v>
+        <f t="shared" si="11"/>
+        <v>4.2210000000000001</v>
       </c>
       <c r="O163" s="12"/>
     </row>
     <row r="164" spans="1:22" ht="24.75" thickBot="1">
+      <c r="A164" s="5"/>
       <c r="B164" s="10">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="B164:B171" si="14">ROW(B164)-ROW($B$2)</f>
         <v>162</v>
       </c>
       <c r="C164" s="11" t="s">
         <v>661</v>
       </c>
       <c r="D164" s="12" t="s">
-        <v>144</v>
+        <v>662</v>
       </c>
       <c r="E164" s="13" t="s">
-        <v>675</v>
-      </c>
-      <c r="F164" s="15"/>
+        <v>694</v>
+      </c>
+      <c r="F164" s="15" t="s">
+        <v>107</v>
+      </c>
       <c r="G164" s="13" t="s">
-        <v>676</v>
+        <v>695</v>
       </c>
       <c r="H164" s="12" t="s">
-        <v>677</v>
+        <v>242</v>
       </c>
       <c r="I164" s="13"/>
-      <c r="J164" s="12"/>
-      <c r="K164" s="12"/>
-      <c r="L164" s="17" t="s">
-        <v>677</v>
-      </c>
-      <c r="M164" s="18"/>
+      <c r="J164" s="12">
+        <v>1</v>
+      </c>
+      <c r="K164" s="12">
+        <f t="shared" si="12"/>
+        <v>3</v>
+      </c>
+      <c r="L164" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="M164" s="18">
+        <v>1.0093000000000001</v>
+      </c>
       <c r="N164" s="18">
-        <f t="shared" ref="N164:N167" si="14">M164*K164</f>
-        <v>0</v>
+        <f>M164*K164</f>
+        <v>3.0279000000000003</v>
       </c>
       <c r="O164" s="12"/>
     </row>
-    <row r="165" spans="1:22" ht="24.75" thickBot="1">
+    <row r="165" spans="1:22" ht="36.75" thickBot="1">
+      <c r="A165" s="5"/>
       <c r="B165" s="10">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>163</v>
       </c>
       <c r="C165" s="11" t="s">
         <v>661</v>
       </c>
       <c r="D165" s="12" t="s">
-        <v>144</v>
+        <v>663</v>
       </c>
       <c r="E165" s="13" t="s">
-        <v>678</v>
-      </c>
-      <c r="F165" s="15"/>
+        <v>664</v>
+      </c>
+      <c r="F165" s="15" t="s">
+        <v>144</v>
+      </c>
       <c r="G165" s="13" t="s">
-        <v>679</v>
+        <v>665</v>
       </c>
       <c r="H165" s="12" t="s">
-        <v>680</v>
-      </c>
-      <c r="I165" s="13"/>
-      <c r="J165" s="12"/>
-      <c r="K165" s="12"/>
+        <v>242</v>
+      </c>
+      <c r="I165" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="J165" s="12">
+        <v>1</v>
+      </c>
+      <c r="K165" s="12">
+        <v>3</v>
+      </c>
       <c r="L165" s="17" t="s">
-        <v>680</v>
-      </c>
-      <c r="M165" s="18"/>
+        <v>110</v>
+      </c>
+      <c r="M165" s="18">
+        <v>0.43</v>
+      </c>
       <c r="N165" s="18">
+        <f>M165*K165</f>
+        <v>1.29</v>
+      </c>
+      <c r="O165" s="12"/>
+    </row>
+    <row r="166" spans="1:22" ht="30.75" thickBot="1">
+      <c r="A166" s="5"/>
+      <c r="B166" s="10">
         <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="O165" s="12"/>
-    </row>
-    <row r="166" spans="1:22" ht="48.75" thickBot="1">
-      <c r="B166" s="10">
-        <f t="shared" si="13"/>
         <v>164</v>
       </c>
       <c r="C166" s="11" t="s">
         <v>661</v>
       </c>
       <c r="D166" s="12" t="s">
-        <v>144</v>
+        <v>666</v>
       </c>
       <c r="E166" s="13" t="s">
-        <v>698</v>
+        <v>667</v>
       </c>
       <c r="F166" s="15" t="s">
         <v>144</v>
       </c>
       <c r="G166" s="13" t="s">
-        <v>699</v>
+        <v>144</v>
       </c>
       <c r="H166" s="12" t="s">
-        <v>144</v>
+        <v>668</v>
       </c>
       <c r="I166" s="13" t="s">
         <v>144</v>
       </c>
       <c r="J166" s="12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K166" s="12">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="L166" s="19" t="s">
         <v>669</v>
       </c>
-      <c r="M166" s="40">
-        <v>2.3199999999999998</v>
+      <c r="M166" s="18">
+        <v>9.8699999999999992</v>
       </c>
       <c r="N166" s="18">
+        <f>M166*K166</f>
+        <v>29.61</v>
+      </c>
+      <c r="O166" s="12"/>
+    </row>
+    <row r="167" spans="1:22" ht="15.75" thickBot="1">
+      <c r="B167" s="10">
         <f t="shared" si="14"/>
-        <v>231.99999999999997</v>
-      </c>
-      <c r="O166" s="12"/>
-      <c r="T166" s="3"/>
-      <c r="U166" s="3"/>
-      <c r="V166" s="3"/>
-    </row>
-    <row r="167" spans="1:22" ht="24.75" thickBot="1">
-      <c r="B167" s="10">
-        <f t="shared" si="13"/>
         <v>165</v>
       </c>
       <c r="C167" s="11" t="s">
         <v>661</v>
       </c>
       <c r="D167" s="12" t="s">
-        <v>144</v>
+        <v>670</v>
       </c>
       <c r="E167" s="13" t="s">
+        <v>671</v>
+      </c>
+      <c r="F167" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G167" s="13" t="s">
+        <v>672</v>
+      </c>
+      <c r="H167" s="12" t="s">
+        <v>673</v>
+      </c>
+      <c r="I167" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="J167" s="12">
+        <v>1</v>
+      </c>
+      <c r="K167" s="12">
+        <v>3</v>
+      </c>
+      <c r="L167" s="19" t="s">
+        <v>674</v>
+      </c>
+      <c r="M167" s="18">
+        <v>99</v>
+      </c>
+      <c r="N167" s="18">
+        <f>M167*K167</f>
+        <v>297</v>
+      </c>
+      <c r="O167" s="12"/>
+    </row>
+    <row r="168" spans="1:22" ht="24.75" thickBot="1">
+      <c r="B168" s="10">
+        <f t="shared" si="14"/>
+        <v>166</v>
+      </c>
+      <c r="C168" s="11" t="s">
+        <v>661</v>
+      </c>
+      <c r="D168" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="E168" s="13" t="s">
+        <v>675</v>
+      </c>
+      <c r="F168" s="15"/>
+      <c r="G168" s="13" t="s">
+        <v>676</v>
+      </c>
+      <c r="H168" s="12" t="s">
+        <v>677</v>
+      </c>
+      <c r="I168" s="13"/>
+      <c r="J168" s="12"/>
+      <c r="K168" s="12"/>
+      <c r="L168" s="17" t="s">
+        <v>677</v>
+      </c>
+      <c r="M168" s="18"/>
+      <c r="N168" s="18">
+        <f t="shared" ref="N168:N171" si="15">M168*K168</f>
+        <v>0</v>
+      </c>
+      <c r="O168" s="12"/>
+    </row>
+    <row r="169" spans="1:22" ht="24.75" thickBot="1">
+      <c r="B169" s="10">
+        <f t="shared" si="14"/>
+        <v>167</v>
+      </c>
+      <c r="C169" s="11" t="s">
+        <v>661</v>
+      </c>
+      <c r="D169" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="E169" s="13" t="s">
+        <v>678</v>
+      </c>
+      <c r="F169" s="15"/>
+      <c r="G169" s="13" t="s">
+        <v>679</v>
+      </c>
+      <c r="H169" s="12" t="s">
+        <v>680</v>
+      </c>
+      <c r="I169" s="13"/>
+      <c r="J169" s="12"/>
+      <c r="K169" s="12"/>
+      <c r="L169" s="17" t="s">
+        <v>680</v>
+      </c>
+      <c r="M169" s="18"/>
+      <c r="N169" s="18">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="O169" s="12"/>
+    </row>
+    <row r="170" spans="1:22" ht="48.75" thickBot="1">
+      <c r="B170" s="10">
+        <f t="shared" si="14"/>
+        <v>168</v>
+      </c>
+      <c r="C170" s="11" t="s">
+        <v>661</v>
+      </c>
+      <c r="D170" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="E170" s="13" t="s">
+        <v>698</v>
+      </c>
+      <c r="F170" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="G170" s="13" t="s">
+        <v>699</v>
+      </c>
+      <c r="H170" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="I170" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="J170" s="12">
+        <v>4</v>
+      </c>
+      <c r="K170" s="12">
+        <v>100</v>
+      </c>
+      <c r="L170" s="19" t="s">
+        <v>669</v>
+      </c>
+      <c r="M170" s="40">
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="N170" s="18">
+        <f t="shared" si="15"/>
+        <v>231.99999999999997</v>
+      </c>
+      <c r="O170" s="12"/>
+      <c r="T170" s="3"/>
+      <c r="U170" s="3"/>
+      <c r="V170" s="3"/>
+    </row>
+    <row r="171" spans="1:22" ht="24.75" thickBot="1">
+      <c r="B171" s="10">
+        <f t="shared" si="14"/>
+        <v>169</v>
+      </c>
+      <c r="C171" s="11" t="s">
+        <v>661</v>
+      </c>
+      <c r="D171" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="E171" s="13" t="s">
         <v>681</v>
       </c>
-      <c r="F167" s="15"/>
-      <c r="G167" s="13" t="s">
+      <c r="F171" s="15"/>
+      <c r="G171" s="13" t="s">
         <v>682</v>
       </c>
-      <c r="H167" s="12" t="s">
+      <c r="H171" s="12" t="s">
         <v>683</v>
       </c>
-      <c r="I167" s="13"/>
-      <c r="J167" s="12"/>
-      <c r="K167" s="12"/>
-      <c r="L167" s="17" t="s">
+      <c r="I171" s="13"/>
+      <c r="J171" s="12"/>
+      <c r="K171" s="12"/>
+      <c r="L171" s="17" t="s">
         <v>684</v>
       </c>
-      <c r="M167" s="40"/>
-      <c r="N167" s="18">
-        <f t="shared" si="14"/>
+      <c r="M171" s="40"/>
+      <c r="N171" s="18">
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="O167" s="12"/>
-    </row>
-    <row r="168" spans="1:22">
-      <c r="M168" s="41" t="s">
+      <c r="O171" s="12"/>
+    </row>
+    <row r="172" spans="1:22">
+      <c r="M172" s="41" t="s">
         <v>685</v>
       </c>
-      <c r="N168" s="42">
-        <f>SUM(N3:N167)</f>
-        <v>1037.1835900000001</v>
-      </c>
-    </row>
-    <row r="169" spans="1:22" ht="15.75" thickBot="1">
-      <c r="M169" s="43" t="s">
+      <c r="N172" s="42">
+        <f>SUM(N3:N171)</f>
+        <v>1043.7025900000001</v>
+      </c>
+    </row>
+    <row r="173" spans="1:22" ht="15.75" thickBot="1">
+      <c r="M173" s="43" t="s">
         <v>686</v>
       </c>
-      <c r="N169" s="44">
-        <f>N168/3</f>
-        <v>345.72786333333335</v>
-      </c>
-    </row>
-    <row r="170" spans="1:22" s="3" customFormat="1">
-      <c r="B170" s="4"/>
-      <c r="C170" s="4"/>
-      <c r="D170"/>
-      <c r="E170"/>
-      <c r="F170"/>
-      <c r="G170"/>
-      <c r="H170"/>
-      <c r="I170"/>
-      <c r="J170"/>
-      <c r="K170"/>
-      <c r="L170"/>
-      <c r="M170"/>
-      <c r="N170"/>
-      <c r="O170"/>
-      <c r="Q170"/>
-      <c r="R170"/>
-      <c r="S170"/>
-      <c r="T170"/>
-      <c r="U170"/>
-      <c r="V170"/>
+      <c r="N173" s="44">
+        <f>N172/3</f>
+        <v>347.90086333333335</v>
+      </c>
+    </row>
+    <row r="174" spans="1:22" s="3" customFormat="1">
+      <c r="B174" s="4"/>
+      <c r="C174" s="4"/>
+      <c r="D174"/>
+      <c r="E174"/>
+      <c r="F174"/>
+      <c r="G174"/>
+      <c r="H174"/>
+      <c r="I174"/>
+      <c r="J174"/>
+      <c r="K174"/>
+      <c r="L174"/>
+      <c r="M174"/>
+      <c r="N174"/>
+      <c r="O174"/>
+      <c r="Q174"/>
+      <c r="R174"/>
+      <c r="S174"/>
+      <c r="T174"/>
+      <c r="U174"/>
+      <c r="V174"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10766,23 +10977,27 @@
     <hyperlink ref="L157" r:id="rId142"/>
     <hyperlink ref="L158" r:id="rId143"/>
     <hyperlink ref="L159" r:id="rId144"/>
-    <hyperlink ref="L165" r:id="rId145"/>
-    <hyperlink ref="L164" r:id="rId146"/>
-    <hyperlink ref="L167" r:id="rId147"/>
-    <hyperlink ref="L162" r:id="rId148"/>
-    <hyperlink ref="L161" r:id="rId149"/>
+    <hyperlink ref="L169" r:id="rId145"/>
+    <hyperlink ref="L168" r:id="rId146"/>
+    <hyperlink ref="L171" r:id="rId147"/>
+    <hyperlink ref="L166" r:id="rId148"/>
+    <hyperlink ref="L165" r:id="rId149"/>
     <hyperlink ref="L56" r:id="rId150"/>
     <hyperlink ref="L71" r:id="rId151"/>
     <hyperlink ref="L133" r:id="rId152"/>
-    <hyperlink ref="L160" r:id="rId153"/>
+    <hyperlink ref="L164" r:id="rId153"/>
     <hyperlink ref="L23" r:id="rId154"/>
-    <hyperlink ref="L166" r:id="rId155"/>
+    <hyperlink ref="L170" r:id="rId155"/>
     <hyperlink ref="L33" r:id="rId156"/>
     <hyperlink ref="L51" r:id="rId157"/>
     <hyperlink ref="L85" r:id="rId158"/>
     <hyperlink ref="L132" r:id="rId159"/>
+    <hyperlink ref="L163" r:id="rId160"/>
+    <hyperlink ref="L160" r:id="rId161"/>
+    <hyperlink ref="L161" r:id="rId162"/>
+    <hyperlink ref="L162" r:id="rId163"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId160"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId164"/>
 </worksheet>
 </file>
</xml_diff>